<commit_message>
combined and error log file
</commit_message>
<xml_diff>
--- a/backend/distribution_live_backup.xlsx
+++ b/backend/distribution_live_backup.xlsx
@@ -6748,22 +6748,22 @@
     </row>
     <row r="266">
       <c r="A266" t="str">
-        <v>1778659312652_99</v>
+        <v>1778659312652_108</v>
       </c>
       <c r="B266" t="str">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="C266" t="str">
-        <v>236</v>
+        <v>588</v>
       </c>
       <c r="D266" t="str">
-        <v>Batul bai Johar bhai Saroda</v>
+        <v>Bilqis bai Husain bhai Gadi</v>
       </c>
       <c r="E266" t="str">
-        <v>30488741</v>
+        <v>20318760</v>
       </c>
       <c r="F266" t="str">
-        <v>Given</v>
+        <v>Pending</v>
       </c>
       <c r="G266" t="str">
         <v/>
@@ -6771,19 +6771,19 @@
     </row>
     <row r="267">
       <c r="A267" t="str">
-        <v>1778659312652_108</v>
+        <v>1778659312652_326</v>
       </c>
       <c r="B267" t="str">
-        <v>109</v>
+        <v>327</v>
       </c>
       <c r="C267" t="str">
-        <v>588</v>
+        <v>431</v>
       </c>
       <c r="D267" t="str">
-        <v>Bilqis bai Husain bhai Gadi</v>
+        <v>Khadija bai Fakhruddin bhai Peeth</v>
       </c>
       <c r="E267" t="str">
-        <v>20318760</v>
+        <v>30366840</v>
       </c>
       <c r="F267" t="str">
         <v>Pending</v>
@@ -6794,25 +6794,34 @@
     </row>
     <row r="268">
       <c r="A268" t="str">
-        <v>1778659312652_326</v>
+        <v>1778659312652_99</v>
       </c>
       <c r="B268" t="str">
-        <v>327</v>
+        <v>100</v>
       </c>
       <c r="C268" t="str">
-        <v>431</v>
+        <v>236</v>
       </c>
       <c r="D268" t="str">
-        <v>Khadija bai Fakhruddin bhai Peeth</v>
+        <v>Batul bai Johar bhai Saroda</v>
       </c>
       <c r="E268" t="str">
-        <v>30366840</v>
+        <v>30488741</v>
       </c>
       <c r="F268" t="str">
-        <v>Pending</v>
+        <v>Given</v>
       </c>
       <c r="G268" t="str">
-        <v/>
+        <v>Ilyas</v>
+      </c>
+      <c r="H268" t="str">
+        <v>19/05/2026</v>
+      </c>
+      <c r="I268" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="J268" t="str">
+        <v>17:29:45</v>
       </c>
     </row>
     <row r="269">

</xml_diff>

<commit_message>
combined and error log file 2
</commit_message>
<xml_diff>
--- a/backend/distribution_live_backup.xlsx
+++ b/backend/distribution_live_backup.xlsx
@@ -6748,42 +6748,51 @@
     </row>
     <row r="266">
       <c r="A266" t="str">
-        <v>1778659312652_108</v>
+        <v>1778659312652_99</v>
       </c>
       <c r="B266" t="str">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="C266" t="str">
-        <v>588</v>
+        <v>236</v>
       </c>
       <c r="D266" t="str">
-        <v>Bilqis bai Husain bhai Gadi</v>
+        <v>Batul bai Johar bhai Saroda</v>
       </c>
       <c r="E266" t="str">
-        <v>20318760</v>
+        <v>30488741</v>
       </c>
       <c r="F266" t="str">
-        <v>Pending</v>
+        <v>Given</v>
       </c>
       <c r="G266" t="str">
-        <v/>
+        <v>Ilya</v>
+      </c>
+      <c r="H266" t="str">
+        <v>19/05/2026</v>
+      </c>
+      <c r="I266" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="J266" t="str">
+        <v>18:22:57</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="str">
-        <v>1778659312652_326</v>
+        <v>1778659312652_108</v>
       </c>
       <c r="B267" t="str">
-        <v>327</v>
+        <v>109</v>
       </c>
       <c r="C267" t="str">
-        <v>431</v>
+        <v>588</v>
       </c>
       <c r="D267" t="str">
-        <v>Khadija bai Fakhruddin bhai Peeth</v>
+        <v>Bilqis bai Husain bhai Gadi</v>
       </c>
       <c r="E267" t="str">
-        <v>30366840</v>
+        <v>20318760</v>
       </c>
       <c r="F267" t="str">
         <v>Pending</v>
@@ -6794,34 +6803,25 @@
     </row>
     <row r="268">
       <c r="A268" t="str">
-        <v>1778659312652_99</v>
+        <v>1778659312652_326</v>
       </c>
       <c r="B268" t="str">
-        <v>100</v>
+        <v>327</v>
       </c>
       <c r="C268" t="str">
-        <v>236</v>
+        <v>431</v>
       </c>
       <c r="D268" t="str">
-        <v>Batul bai Johar bhai Saroda</v>
+        <v>Khadija bai Fakhruddin bhai Peeth</v>
       </c>
       <c r="E268" t="str">
-        <v>30488741</v>
+        <v>30366840</v>
       </c>
       <c r="F268" t="str">
-        <v>Given</v>
+        <v>Pending</v>
       </c>
       <c r="G268" t="str">
-        <v>Ilyas</v>
-      </c>
-      <c r="H268" t="str">
-        <v>19/05/2026</v>
-      </c>
-      <c r="I268" t="str">
-        <v>Tuesday</v>
-      </c>
-      <c r="J268" t="str">
-        <v>17:29:45</v>
+        <v/>
       </c>
     </row>
     <row r="269">

</xml_diff>

<commit_message>
Full Software Design Change Another section Bulk Distribution Entry
</commit_message>
<xml_diff>
--- a/backend/distribution_live_backup.xlsx
+++ b/backend/distribution_live_backup.xlsx
@@ -1219,19 +1219,10 @@
         <v>20387894</v>
       </c>
       <c r="F32" t="str">
-        <v>Given</v>
+        <v>Pending</v>
       </c>
       <c r="G32" t="str">
-        <v>Ilyas</v>
-      </c>
-      <c r="H32" t="str">
-        <v>24/05/2026</v>
-      </c>
-      <c r="I32" t="str">
-        <v>Sunday</v>
-      </c>
-      <c r="J32" t="str">
-        <v>20:53:42</v>
+        <v/>
       </c>
     </row>
     <row r="33">
@@ -1259,88 +1250,97 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>1778659312652_145</v>
+        <v>1778659312652_154</v>
       </c>
       <c r="B34" t="str">
-        <v>146</v>
+        <v>155</v>
       </c>
       <c r="C34" t="str">
-        <v>1234</v>
+        <v>1339</v>
       </c>
       <c r="D34" t="str">
-        <v>Fakhruddin bhai Talib bhai Najafi</v>
+        <v>Farida bai Mohammedhusain bhai Kothari</v>
       </c>
       <c r="E34" t="str">
-        <v>30368536</v>
+        <v>30367383</v>
       </c>
       <c r="F34" t="str">
-        <v>Pending</v>
+        <v>Given</v>
       </c>
       <c r="G34" t="str">
-        <v/>
+        <v>Ilyas</v>
+      </c>
+      <c r="H34" t="str">
+        <v>24/05/2026</v>
+      </c>
+      <c r="I34" t="str">
+        <v>Sunday</v>
+      </c>
+      <c r="J34" t="str">
+        <v>22:35:04</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>1778659312652_146</v>
+        <v>1778659312652_145</v>
       </c>
       <c r="B35" t="str">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C35" t="str">
-        <v>855</v>
+        <v>1234</v>
       </c>
       <c r="D35" t="str">
-        <v>Fakhruddin bhai Yusuf bhai Kabja</v>
+        <v>Fakhruddin bhai Talib bhai Najafi</v>
       </c>
       <c r="E35" t="str">
-        <v>30367601</v>
+        <v>30368536</v>
       </c>
       <c r="F35" t="str">
-        <v>Given</v>
+        <v>Pending</v>
       </c>
       <c r="G35" t="str">
-        <v>Fakhruddin kawja</v>
+        <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>1778659312652_14</v>
+        <v>1778659312652_146</v>
       </c>
       <c r="B36" t="str">
-        <v>15</v>
+        <v>147</v>
       </c>
       <c r="C36" t="str">
-        <v>1452</v>
+        <v>855</v>
       </c>
       <c r="D36" t="str">
-        <v>Abdeali bhai Husain bhai Kika</v>
+        <v>Fakhruddin bhai Yusuf bhai Kabja</v>
       </c>
       <c r="E36" t="str">
-        <v>30367463</v>
+        <v>30367601</v>
       </c>
       <c r="F36" t="str">
-        <v>Pending</v>
+        <v>Given</v>
       </c>
       <c r="G36" t="str">
-        <v/>
+        <v>Fakhruddin kawja</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>1778659312652_149</v>
+        <v>1778659312652_14</v>
       </c>
       <c r="B37" t="str">
-        <v>150</v>
+        <v>15</v>
       </c>
       <c r="C37" t="str">
-        <v>315</v>
+        <v>1452</v>
       </c>
       <c r="D37" t="str">
-        <v>Farida bai Fakhruddin bhai Rustam</v>
+        <v>Abdeali bhai Husain bhai Kika</v>
       </c>
       <c r="E37" t="str">
-        <v>20318201</v>
+        <v>30367463</v>
       </c>
       <c r="F37" t="str">
         <v>Pending</v>
@@ -1351,74 +1351,74 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>1778659312652_150</v>
+        <v>1778659312652_149</v>
       </c>
       <c r="B38" t="str">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C38" t="str">
-        <v>491</v>
+        <v>315</v>
       </c>
       <c r="D38" t="str">
-        <v>Farida bai Husain bhai Galalji</v>
+        <v>Farida bai Fakhruddin bhai Rustam</v>
       </c>
       <c r="E38" t="str">
-        <v>30366897</v>
+        <v>20318201</v>
       </c>
       <c r="F38" t="str">
-        <v>Given</v>
+        <v>Pending</v>
       </c>
       <c r="G38" t="str">
-        <v>Zainab ben shabbir bhai Dhambola</v>
-      </c>
-      <c r="H38" t="str">
-        <v>22/05/2026</v>
-      </c>
-      <c r="I38" t="str">
-        <v>Friday</v>
-      </c>
-      <c r="J38" t="str">
-        <v>11:31:37</v>
+        <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>1778659312652_151</v>
+        <v>1778659312652_150</v>
       </c>
       <c r="B39" t="str">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C39" t="str">
-        <v>1122</v>
+        <v>491</v>
       </c>
       <c r="D39" t="str">
-        <v>Farida bai Juzer bhai Gyori</v>
+        <v>Farida bai Husain bhai Galalji</v>
       </c>
       <c r="E39" t="str">
-        <v>30367320</v>
+        <v>30366897</v>
       </c>
       <c r="F39" t="str">
-        <v>Pending</v>
+        <v>Given</v>
       </c>
       <c r="G39" t="str">
-        <v/>
+        <v>Zainab ben shabbir bhai Dhambola</v>
+      </c>
+      <c r="H39" t="str">
+        <v>22/05/2026</v>
+      </c>
+      <c r="I39" t="str">
+        <v>Friday</v>
+      </c>
+      <c r="J39" t="str">
+        <v>11:31:37</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>1778659312652_152</v>
+        <v>1778659312652_151</v>
       </c>
       <c r="B40" t="str">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C40" t="str">
-        <v>970</v>
+        <v>1122</v>
       </c>
       <c r="D40" t="str">
-        <v>Farida bai Khuzaima bhai Obri</v>
+        <v>Farida bai Juzer bhai Gyori</v>
       </c>
       <c r="E40" t="str">
-        <v>30367525</v>
+        <v>30367320</v>
       </c>
       <c r="F40" t="str">
         <v>Pending</v>
@@ -1429,19 +1429,19 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>1778659312652_153</v>
+        <v>1778659312652_152</v>
       </c>
       <c r="B41" t="str">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C41" t="str">
-        <v>1336</v>
+        <v>970</v>
       </c>
       <c r="D41" t="str">
-        <v>Farida bai Mohammed bhai Maudiwala</v>
+        <v>Farida bai Khuzaima bhai Obri</v>
       </c>
       <c r="E41" t="str">
-        <v>30367788</v>
+        <v>30367525</v>
       </c>
       <c r="F41" t="str">
         <v>Pending</v>
@@ -1452,66 +1452,57 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>1778659312652_391</v>
+        <v>1778659312652_153</v>
       </c>
       <c r="B42" t="str">
-        <v>392</v>
+        <v>154</v>
       </c>
       <c r="C42" t="str">
-        <v>1055</v>
+        <v>1336</v>
       </c>
       <c r="D42" t="str">
-        <v>Mulla Husain bhai Jivaji bhai Pachlasa</v>
+        <v>Farida bai Mohammed bhai Maudiwala</v>
       </c>
       <c r="E42" t="str">
-        <v>20318738</v>
+        <v>30367788</v>
       </c>
       <c r="F42" t="str">
-        <v>Given</v>
+        <v>Pending</v>
       </c>
       <c r="G42" t="str">
         <v/>
-      </c>
-      <c r="H42" t="str">
-        <v>22/05/2026</v>
-      </c>
-      <c r="I42" t="str">
-        <v>Friday</v>
-      </c>
-      <c r="J42" t="str">
-        <v>11:46:17</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>1778659312652_154</v>
+        <v>1778659312652_391</v>
       </c>
       <c r="B43" t="str">
-        <v>155</v>
+        <v>392</v>
       </c>
       <c r="C43" t="str">
-        <v>1339</v>
+        <v>1055</v>
       </c>
       <c r="D43" t="str">
-        <v>Farida bai Mohammedhusain bhai Kothari</v>
+        <v>Mulla Husain bhai Jivaji bhai Pachlasa</v>
       </c>
       <c r="E43" t="str">
-        <v>30367383</v>
+        <v>20318738</v>
       </c>
       <c r="F43" t="str">
         <v>Given</v>
       </c>
       <c r="G43" t="str">
-        <v>Ilyas</v>
+        <v/>
       </c>
       <c r="H43" t="str">
-        <v>16/05/2026</v>
+        <v>22/05/2026</v>
       </c>
       <c r="I43" t="str">
-        <v>Saturday</v>
+        <v>Friday</v>
       </c>
       <c r="J43" t="str">
-        <v>11:45:49</v>
+        <v>11:46:17</v>
       </c>
     </row>
     <row r="44">
@@ -5055,106 +5046,97 @@
     </row>
     <row r="183">
       <c r="A183" t="str">
-        <v>1778659312652_575</v>
+        <v>1778659312652_219</v>
       </c>
       <c r="B183" t="str">
-        <v>576</v>
+        <v>220</v>
       </c>
       <c r="C183" t="str">
-        <v>238</v>
+        <v>813</v>
       </c>
       <c r="D183" t="str">
-        <v>Samina bai Husain bhai Hathai</v>
+        <v>Fatema bai Saifuddin bhai Khand</v>
       </c>
       <c r="E183" t="str">
-        <v>20318771</v>
+        <v>20318516</v>
       </c>
       <c r="F183" t="str">
         <v>Given</v>
       </c>
       <c r="G183" t="str">
-        <v>Ilyas</v>
-      </c>
-      <c r="H183" t="str">
-        <v>24/05/2026</v>
-      </c>
-      <c r="I183" t="str">
-        <v>Sunday</v>
-      </c>
-      <c r="J183" t="str">
-        <v>20:53:42</v>
+        <v>Fakhruddin kawja</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="str">
-        <v>1778659312652_219</v>
+        <v>1778659312652_220</v>
       </c>
       <c r="B184" t="str">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C184" t="str">
-        <v>813</v>
+        <v>415</v>
       </c>
       <c r="D184" t="str">
-        <v>Fatema bai Saifuddin bhai Khand</v>
+        <v>Fatema bai Saifuddin bhai Morawala</v>
       </c>
       <c r="E184" t="str">
-        <v>20318516</v>
+        <v>30366819</v>
       </c>
       <c r="F184" t="str">
         <v>Given</v>
       </c>
       <c r="G184" t="str">
-        <v>Fakhruddin kawja</v>
+        <v>shkh fakhruddin badi</v>
+      </c>
+      <c r="H184" t="str">
+        <v>19/05/2026</v>
+      </c>
+      <c r="I184" t="str">
+        <v>Tuesday</v>
+      </c>
+      <c r="J184" t="str">
+        <v>11:29:18</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="str">
-        <v>1778659312652_220</v>
+        <v>1778659312652_241</v>
       </c>
       <c r="B185" t="str">
-        <v>221</v>
+        <v>242</v>
       </c>
       <c r="C185" t="str">
-        <v>415</v>
+        <v>874</v>
       </c>
       <c r="D185" t="str">
-        <v>Fatema bai Saifuddin bhai Morawala</v>
+        <v>Ghulamabbas bhai Mulla Fidahusain bhai Baroda</v>
       </c>
       <c r="E185" t="str">
-        <v>30366819</v>
+        <v>20318553</v>
       </c>
       <c r="F185" t="str">
-        <v>Given</v>
+        <v>Pending</v>
       </c>
       <c r="G185" t="str">
-        <v>shkh fakhruddin badi</v>
-      </c>
-      <c r="H185" t="str">
-        <v>19/05/2026</v>
-      </c>
-      <c r="I185" t="str">
-        <v>Tuesday</v>
-      </c>
-      <c r="J185" t="str">
-        <v>11:29:18</v>
+        <v/>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="str">
-        <v>1778659312652_241</v>
+        <v>1778659312652_413</v>
       </c>
       <c r="B186" t="str">
-        <v>242</v>
+        <v>414</v>
       </c>
       <c r="C186" t="str">
-        <v>874</v>
+        <v/>
       </c>
       <c r="D186" t="str">
-        <v>Ghulamabbas bhai Mulla Fidahusain bhai Baroda</v>
+        <v>Mustafa bhai Hakimuddin bhai Lodal</v>
       </c>
       <c r="E186" t="str">
-        <v>20318553</v>
+        <v>30493059</v>
       </c>
       <c r="F186" t="str">
         <v>Pending</v>
@@ -5165,19 +5147,19 @@
     </row>
     <row r="187">
       <c r="A187" t="str">
-        <v>1778659312652_413</v>
+        <v>1778659312652_414</v>
       </c>
       <c r="B187" t="str">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="C187" t="str">
         <v/>
       </c>
       <c r="D187" t="str">
-        <v>Mustafa bhai Hakimuddin bhai Lodal</v>
+        <v>Mustafa bhai Taher bhai Bapu</v>
       </c>
       <c r="E187" t="str">
-        <v>30493059</v>
+        <v>20318039</v>
       </c>
       <c r="F187" t="str">
         <v>Pending</v>
@@ -5188,19 +5170,19 @@
     </row>
     <row r="188">
       <c r="A188" t="str">
-        <v>1778659312652_414</v>
+        <v>1778659312652_415</v>
       </c>
       <c r="B188" t="str">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C188" t="str">
-        <v/>
+        <v>52</v>
       </c>
       <c r="D188" t="str">
-        <v>Mustafa bhai Taher bhai Bapu</v>
+        <v>Mustansir bhai Abbas bhai Ramakda</v>
       </c>
       <c r="E188" t="str">
-        <v>20318039</v>
+        <v>30805007</v>
       </c>
       <c r="F188" t="str">
         <v>Pending</v>
@@ -5211,175 +5193,175 @@
     </row>
     <row r="189">
       <c r="A189" t="str">
-        <v>1778659312652_415</v>
+        <v>1778659312652_446</v>
       </c>
       <c r="B189" t="str">
-        <v>416</v>
+        <v>447</v>
       </c>
       <c r="C189" t="str">
-        <v>52</v>
+        <v>442</v>
       </c>
       <c r="D189" t="str">
-        <v>Mustansir bhai Abbas bhai Ramakda</v>
+        <v>Qaidjoher bhai Shabbirhusain bhai Ramgarh</v>
       </c>
       <c r="E189" t="str">
-        <v>30805007</v>
+        <v>20342316</v>
       </c>
       <c r="F189" t="str">
-        <v>Pending</v>
+        <v>Given</v>
       </c>
       <c r="G189" t="str">
-        <v/>
+        <v>Nasa bhai</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="str">
-        <v>1778659312652_446</v>
+        <v>1778659312652_447</v>
       </c>
       <c r="B190" t="str">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="C190" t="str">
-        <v>442</v>
+        <v>1360</v>
       </c>
       <c r="D190" t="str">
-        <v>Qaidjoher bhai Shabbirhusain bhai Ramgarh</v>
+        <v>Qaidjoher bhai Shaikh Abbas bhai Kothra</v>
       </c>
       <c r="E190" t="str">
-        <v>20342316</v>
+        <v>20406019</v>
       </c>
       <c r="F190" t="str">
-        <v>Given</v>
+        <v>Pending</v>
       </c>
       <c r="G190" t="str">
-        <v>Nasa bhai</v>
+        <v/>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="str">
-        <v>1778659312652_447</v>
+        <v>1778659312652_21</v>
       </c>
       <c r="B191" t="str">
-        <v>448</v>
+        <v>22</v>
       </c>
       <c r="C191" t="str">
-        <v>1360</v>
+        <v>789</v>
       </c>
       <c r="D191" t="str">
-        <v>Qaidjoher bhai Shaikh Abbas bhai Kothra</v>
+        <v>Ajab bai Fakhruddin bhai Wardawala</v>
       </c>
       <c r="E191" t="str">
-        <v>20406019</v>
+        <v>30367453</v>
       </c>
       <c r="F191" t="str">
-        <v>Pending</v>
+        <v>Given</v>
       </c>
       <c r="G191" t="str">
         <v/>
+      </c>
+      <c r="H191" t="str">
+        <v>20/05/2026</v>
+      </c>
+      <c r="I191" t="str">
+        <v>Wednesday</v>
+      </c>
+      <c r="J191" t="str">
+        <v>12:24:47</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="str">
-        <v>1778659312652_21</v>
+        <v>1778659312652_448</v>
       </c>
       <c r="B192" t="str">
-        <v>22</v>
+        <v>449</v>
       </c>
       <c r="C192" t="str">
-        <v>789</v>
+        <v>393</v>
       </c>
       <c r="D192" t="str">
-        <v>Ajab bai Fakhruddin bhai Wardawala</v>
+        <v>Qasimali bhai Taiyebali bhai Kotwal</v>
       </c>
       <c r="E192" t="str">
-        <v>30367453</v>
+        <v>20401345</v>
       </c>
       <c r="F192" t="str">
-        <v>Given</v>
+        <v>Pending</v>
       </c>
       <c r="G192" t="str">
         <v/>
-      </c>
-      <c r="H192" t="str">
-        <v>20/05/2026</v>
-      </c>
-      <c r="I192" t="str">
-        <v>Wednesday</v>
-      </c>
-      <c r="J192" t="str">
-        <v>12:24:47</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="str">
-        <v>1778659312652_448</v>
+        <v>1778659312652_44</v>
       </c>
       <c r="B193" t="str">
-        <v>449</v>
+        <v>45</v>
       </c>
       <c r="C193" t="str">
-        <v>393</v>
+        <v>213</v>
       </c>
       <c r="D193" t="str">
-        <v>Qasimali bhai Taiyebali bhai Kotwal</v>
+        <v>Alefiyah bai Abbasali bhai Fakhri</v>
       </c>
       <c r="E193" t="str">
-        <v>20401345</v>
+        <v>30366726</v>
       </c>
       <c r="F193" t="str">
-        <v>Pending</v>
+        <v>Given</v>
       </c>
       <c r="G193" t="str">
-        <v/>
+        <v>shkh fakhruddin badi</v>
+      </c>
+      <c r="H193" t="str">
+        <v>18/05/2026</v>
+      </c>
+      <c r="I193" t="str">
+        <v>Monday</v>
+      </c>
+      <c r="J193" t="str">
+        <v>11:33:17</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="str">
-        <v>1778659312652_44</v>
+        <v>1778659312652_449</v>
       </c>
       <c r="B194" t="str">
-        <v>45</v>
+        <v>450</v>
       </c>
       <c r="C194" t="str">
-        <v>213</v>
+        <v>1497</v>
       </c>
       <c r="D194" t="str">
-        <v>Alefiyah bai Abbasali bhai Fakhri</v>
+        <v>Quraish bhai Shaikh Mohammed bhai Maharaj</v>
       </c>
       <c r="E194" t="str">
-        <v>30366726</v>
+        <v>20387792</v>
       </c>
       <c r="F194" t="str">
-        <v>Given</v>
+        <v>Pending</v>
       </c>
       <c r="G194" t="str">
-        <v>shkh fakhruddin badi</v>
-      </c>
-      <c r="H194" t="str">
-        <v>18/05/2026</v>
-      </c>
-      <c r="I194" t="str">
-        <v>Monday</v>
-      </c>
-      <c r="J194" t="str">
-        <v>11:33:17</v>
+        <v/>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="str">
-        <v>1778659312652_449</v>
+        <v>1778659312652_575</v>
       </c>
       <c r="B195" t="str">
-        <v>450</v>
+        <v>576</v>
       </c>
       <c r="C195" t="str">
-        <v>1497</v>
+        <v>238</v>
       </c>
       <c r="D195" t="str">
-        <v>Quraish bhai Shaikh Mohammed bhai Maharaj</v>
+        <v>Samina bai Husain bhai Hathai</v>
       </c>
       <c r="E195" t="str">
-        <v>20387792</v>
+        <v>20318771</v>
       </c>
       <c r="F195" t="str">
         <v>Pending</v>
@@ -7042,51 +7024,42 @@
     </row>
     <row r="260">
       <c r="A260" t="str">
-        <v>1778659312652_99</v>
+        <v>1778659312652_103</v>
       </c>
       <c r="B260" t="str">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C260" t="str">
-        <v>236</v>
+        <v>1303</v>
       </c>
       <c r="D260" t="str">
-        <v>Batul bai Johar bhai Saroda</v>
+        <v>Batul bai Qutbuddin bhai Rustam</v>
       </c>
       <c r="E260" t="str">
-        <v>30488741</v>
+        <v>30366656</v>
       </c>
       <c r="F260" t="str">
-        <v>Given</v>
+        <v>Pending</v>
       </c>
       <c r="G260" t="str">
-        <v>Ilyas</v>
-      </c>
-      <c r="H260" t="str">
-        <v>24/05/2026</v>
-      </c>
-      <c r="I260" t="str">
-        <v>Sunday</v>
-      </c>
-      <c r="J260" t="str">
-        <v>20:29:18</v>
+        <v/>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="str">
-        <v>1778659312652_103</v>
+        <v>1778659312652_104</v>
       </c>
       <c r="B261" t="str">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C261" t="str">
-        <v>1303</v>
+        <v>76</v>
       </c>
       <c r="D261" t="str">
-        <v>Batul bai Qutbuddin bhai Rustam</v>
+        <v>Batul bai Saifuddin bhai Doodhbhai</v>
       </c>
       <c r="E261" t="str">
-        <v>30366656</v>
+        <v>30368616</v>
       </c>
       <c r="F261" t="str">
         <v>Pending</v>
@@ -7097,19 +7070,19 @@
     </row>
     <row r="262">
       <c r="A262" t="str">
-        <v>1778659312652_104</v>
+        <v>1778659312652_105</v>
       </c>
       <c r="B262" t="str">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C262" t="str">
-        <v>76</v>
+        <v>744</v>
       </c>
       <c r="D262" t="str">
-        <v>Batul bai Saifuddin bhai Doodhbhai</v>
+        <v>Batul bai Shaikh Akbarhusain bhai Rampurwala</v>
       </c>
       <c r="E262" t="str">
-        <v>30368616</v>
+        <v>30367359</v>
       </c>
       <c r="F262" t="str">
         <v>Pending</v>
@@ -7120,80 +7093,89 @@
     </row>
     <row r="263">
       <c r="A263" t="str">
-        <v>1778659312652_105</v>
+        <v>1778659312652_106</v>
       </c>
       <c r="B263" t="str">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C263" t="str">
-        <v>744</v>
+        <v>807</v>
       </c>
       <c r="D263" t="str">
-        <v>Batul bai Shaikh Akbarhusain bhai Rampurwala</v>
+        <v>Batul bai Taiyebali bhai Bankoda</v>
       </c>
       <c r="E263" t="str">
-        <v>30367359</v>
+        <v>30367508</v>
       </c>
       <c r="F263" t="str">
-        <v>Pending</v>
+        <v>Given</v>
       </c>
       <c r="G263" t="str">
-        <v/>
+        <v>zainab ben antri</v>
+      </c>
+      <c r="H263" t="str">
+        <v>18/05/2026</v>
+      </c>
+      <c r="I263" t="str">
+        <v>Monday</v>
+      </c>
+      <c r="J263" t="str">
+        <v>11:50:34</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="str">
-        <v>1778659312652_106</v>
+        <v>1778659312652_6</v>
       </c>
       <c r="B264" t="str">
-        <v>107</v>
+        <v>7</v>
       </c>
       <c r="C264" t="str">
-        <v>807</v>
+        <v>7</v>
       </c>
       <c r="D264" t="str">
-        <v>Batul bai Taiyebali bhai Bankoda</v>
+        <v>Abbas bhai Alihusain bhai Sihjee</v>
       </c>
       <c r="E264" t="str">
-        <v>30367508</v>
+        <v>20435003</v>
       </c>
       <c r="F264" t="str">
         <v>Given</v>
       </c>
       <c r="G264" t="str">
-        <v>zainab ben antri</v>
+        <v>Ajab ben Khand</v>
       </c>
       <c r="H264" t="str">
-        <v>18/05/2026</v>
+        <v>21/05/2026</v>
       </c>
       <c r="I264" t="str">
-        <v>Monday</v>
+        <v>Thursday</v>
       </c>
       <c r="J264" t="str">
-        <v>11:50:34</v>
+        <v>10:25:43</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="str">
-        <v>1778659312652_6</v>
+        <v>1778659312652_335</v>
       </c>
       <c r="B265" t="str">
-        <v>7</v>
+        <v>336</v>
       </c>
       <c r="C265" t="str">
-        <v>7</v>
+        <v>1197</v>
       </c>
       <c r="D265" t="str">
-        <v>Abbas bhai Alihusain bhai Sihjee</v>
+        <v>Khanali bhai Mohammadhussain bhai Hedari</v>
       </c>
       <c r="E265" t="str">
-        <v>20435003</v>
+        <v>20414120</v>
       </c>
       <c r="F265" t="str">
         <v>Given</v>
       </c>
       <c r="G265" t="str">
-        <v>Ajab ben Khand</v>
+        <v/>
       </c>
       <c r="H265" t="str">
         <v>21/05/2026</v>
@@ -7202,56 +7184,47 @@
         <v>Thursday</v>
       </c>
       <c r="J265" t="str">
-        <v>10:25:43</v>
+        <v>11:08:30</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="str">
-        <v>1778659312652_335</v>
+        <v>1778659312652_107</v>
       </c>
       <c r="B266" t="str">
-        <v>336</v>
+        <v>108</v>
       </c>
       <c r="C266" t="str">
-        <v>1197</v>
+        <v>17</v>
       </c>
       <c r="D266" t="str">
-        <v>Khanali bhai Mohammadhussain bhai Hedari</v>
+        <v>Bilqis bai Abidhusain bhai Nareli</v>
       </c>
       <c r="E266" t="str">
-        <v>20414120</v>
+        <v>20318722</v>
       </c>
       <c r="F266" t="str">
-        <v>Given</v>
+        <v>Pending</v>
       </c>
       <c r="G266" t="str">
         <v/>
-      </c>
-      <c r="H266" t="str">
-        <v>21/05/2026</v>
-      </c>
-      <c r="I266" t="str">
-        <v>Thursday</v>
-      </c>
-      <c r="J266" t="str">
-        <v>11:08:30</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="str">
-        <v>1778659312652_107</v>
+        <v>1778659312652_108</v>
       </c>
       <c r="B267" t="str">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C267" t="str">
-        <v>17</v>
+        <v>588</v>
       </c>
       <c r="D267" t="str">
-        <v>Bilqis bai Abidhusain bhai Nareli</v>
+        <v>Bilqis bai Husain bhai Gadi</v>
       </c>
       <c r="E267" t="str">
-        <v>20318722</v>
+        <v>20318760</v>
       </c>
       <c r="F267" t="str">
         <v>Pending</v>
@@ -7262,19 +7235,19 @@
     </row>
     <row r="268">
       <c r="A268" t="str">
-        <v>1778659312652_108</v>
+        <v>1778659312652_326</v>
       </c>
       <c r="B268" t="str">
-        <v>109</v>
+        <v>327</v>
       </c>
       <c r="C268" t="str">
-        <v>588</v>
+        <v>431</v>
       </c>
       <c r="D268" t="str">
-        <v>Bilqis bai Husain bhai Gadi</v>
+        <v>Khadija bai Fakhruddin bhai Peeth</v>
       </c>
       <c r="E268" t="str">
-        <v>20318760</v>
+        <v>30366840</v>
       </c>
       <c r="F268" t="str">
         <v>Pending</v>
@@ -7285,19 +7258,19 @@
     </row>
     <row r="269">
       <c r="A269" t="str">
-        <v>1778659312652_326</v>
+        <v>1778659312652_327</v>
       </c>
       <c r="B269" t="str">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C269" t="str">
-        <v>431</v>
+        <v>822</v>
       </c>
       <c r="D269" t="str">
-        <v>Khadija bai Fakhruddin bhai Peeth</v>
+        <v>Khadija bai Ghulamhusain bhai Dudhwala</v>
       </c>
       <c r="E269" t="str">
-        <v>30366840</v>
+        <v>30367535</v>
       </c>
       <c r="F269" t="str">
         <v>Pending</v>
@@ -7308,19 +7281,19 @@
     </row>
     <row r="270">
       <c r="A270" t="str">
-        <v>1778659312652_327</v>
+        <v>1778659312652_328</v>
       </c>
       <c r="B270" t="str">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C270" t="str">
-        <v>822</v>
+        <v>684</v>
       </c>
       <c r="D270" t="str">
-        <v>Khadija bai Ghulamhusain bhai Dudhwala</v>
+        <v>Khadija bai Haiderali bhai Maudi wala</v>
       </c>
       <c r="E270" t="str">
-        <v>30367535</v>
+        <v>30367251</v>
       </c>
       <c r="F270" t="str">
         <v>Pending</v>
@@ -7331,19 +7304,19 @@
     </row>
     <row r="271">
       <c r="A271" t="str">
-        <v>1778659312652_328</v>
+        <v>1778659312652_329</v>
       </c>
       <c r="B271" t="str">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C271" t="str">
-        <v>684</v>
+        <v>62</v>
       </c>
       <c r="D271" t="str">
-        <v>Khadija bai Haiderali bhai Maudi wala</v>
+        <v>Khadija bai Mulla Fakhruddin bhai Baroda</v>
       </c>
       <c r="E271" t="str">
-        <v>30367251</v>
+        <v>20318054</v>
       </c>
       <c r="F271" t="str">
         <v>Pending</v>
@@ -7354,97 +7327,97 @@
     </row>
     <row r="272">
       <c r="A272" t="str">
-        <v>1778659312652_329</v>
+        <v>1778659312652_102</v>
       </c>
       <c r="B272" t="str">
-        <v>330</v>
+        <v>103</v>
       </c>
       <c r="C272" t="str">
-        <v>62</v>
+        <v>637</v>
       </c>
       <c r="D272" t="str">
-        <v>Khadija bai Mulla Fakhruddin bhai Baroda</v>
+        <v>Batul bai Mufaddal bhai Jaan</v>
       </c>
       <c r="E272" t="str">
-        <v>20318054</v>
+        <v>30367654</v>
       </c>
       <c r="F272" t="str">
-        <v>Pending</v>
+        <v>Given</v>
       </c>
       <c r="G272" t="str">
-        <v/>
+        <v>mulla jivaji</v>
+      </c>
+      <c r="H272" t="str">
+        <v>22/05/2026</v>
+      </c>
+      <c r="I272" t="str">
+        <v>Friday</v>
+      </c>
+      <c r="J272" t="str">
+        <v>11:47:31</v>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="str">
-        <v>1778659312652_102</v>
+        <v>1778659312652_330</v>
       </c>
       <c r="B273" t="str">
-        <v>103</v>
+        <v>331</v>
       </c>
       <c r="C273" t="str">
-        <v>637</v>
+        <v>1356</v>
       </c>
       <c r="D273" t="str">
-        <v>Batul bai Mufaddal bhai Jaan</v>
+        <v>Khadija bai Murtaza bhai Ratawala</v>
       </c>
       <c r="E273" t="str">
-        <v>30367654</v>
+        <v>30367899</v>
       </c>
       <c r="F273" t="str">
         <v>Given</v>
       </c>
       <c r="G273" t="str">
-        <v>mulla jivaji</v>
-      </c>
-      <c r="H273" t="str">
-        <v>22/05/2026</v>
-      </c>
-      <c r="I273" t="str">
-        <v>Friday</v>
-      </c>
-      <c r="J273" t="str">
-        <v>11:47:31</v>
+        <v>Fakhruddin kawja</v>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="str">
-        <v>1778659312652_330</v>
+        <v>1778659312652_331</v>
       </c>
       <c r="B274" t="str">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C274" t="str">
-        <v>1356</v>
+        <v>388</v>
       </c>
       <c r="D274" t="str">
-        <v>Khadija bai Murtaza bhai Ratawala</v>
+        <v>Khadija bai Qutbuddin bhai Tara</v>
       </c>
       <c r="E274" t="str">
-        <v>30367899</v>
+        <v>30366583</v>
       </c>
       <c r="F274" t="str">
-        <v>Given</v>
+        <v>Pending</v>
       </c>
       <c r="G274" t="str">
-        <v>Fakhruddin kawja</v>
+        <v/>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="str">
-        <v>1778659312652_331</v>
+        <v>1778659312652_332</v>
       </c>
       <c r="B275" t="str">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C275" t="str">
-        <v>388</v>
+        <v>310</v>
       </c>
       <c r="D275" t="str">
-        <v>Khadija bai Qutbuddin bhai Tara</v>
+        <v>Khadija bai Saifuddin bhai Ezzi</v>
       </c>
       <c r="E275" t="str">
-        <v>30366583</v>
+        <v>30366643</v>
       </c>
       <c r="F275" t="str">
         <v>Pending</v>
@@ -7455,114 +7428,114 @@
     </row>
     <row r="276">
       <c r="A276" t="str">
-        <v>1778659312652_332</v>
+        <v>1778659312652_333</v>
       </c>
       <c r="B276" t="str">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C276" t="str">
-        <v>310</v>
+        <v>1029</v>
       </c>
       <c r="D276" t="str">
-        <v>Khadija bai Saifuddin bhai Ezzi</v>
+        <v>Khadija bai Shaikh Mohammed bhai Khumanpur</v>
       </c>
       <c r="E276" t="str">
-        <v>30366643</v>
+        <v>30367849</v>
       </c>
       <c r="F276" t="str">
-        <v>Pending</v>
+        <v>Given</v>
       </c>
       <c r="G276" t="str">
-        <v/>
+        <v>yakut bhai gaba</v>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="str">
-        <v>1778659312652_333</v>
+        <v>1778659312652_334</v>
       </c>
       <c r="B277" t="str">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C277" t="str">
-        <v>1029</v>
+        <v>138</v>
       </c>
       <c r="D277" t="str">
-        <v>Khadija bai Shaikh Mohammed bhai Khumanpur</v>
+        <v>Khadija bai Tayyeb bhai Gadi</v>
       </c>
       <c r="E277" t="str">
-        <v>30367849</v>
+        <v>30366336</v>
       </c>
       <c r="F277" t="str">
         <v>Given</v>
       </c>
       <c r="G277" t="str">
-        <v>yakut bhai gaba</v>
+        <v>shkh fakhruddin badi</v>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="str">
-        <v>1778659312652_334</v>
+        <v>1778659312652_336</v>
       </c>
       <c r="B278" t="str">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="C278" t="str">
-        <v>138</v>
+        <v>980</v>
       </c>
       <c r="D278" t="str">
-        <v>Khadija bai Tayyeb bhai Gadi</v>
+        <v>Khuzaima bhai Shabbirhusain bhai Ramgarhwala</v>
       </c>
       <c r="E278" t="str">
-        <v>30366336</v>
+        <v>20402290</v>
       </c>
       <c r="F278" t="str">
         <v>Given</v>
       </c>
       <c r="G278" t="str">
-        <v>shkh fakhruddin badi</v>
+        <v>Nasa bhai</v>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="str">
-        <v>1778659312652_336</v>
+        <v>1778659312652_698</v>
       </c>
       <c r="B279" t="str">
-        <v>337</v>
+        <v>699</v>
       </c>
       <c r="C279" t="str">
-        <v>980</v>
+        <v>1475</v>
       </c>
       <c r="D279" t="str">
-        <v>Khuzaima bhai Shabbirhusain bhai Ramgarhwala</v>
+        <v>Tasneem bai Yusuf bhai Rail</v>
       </c>
       <c r="E279" t="str">
-        <v>20402290</v>
+        <v>30366367</v>
       </c>
       <c r="F279" t="str">
         <v>Given</v>
       </c>
       <c r="G279" t="str">
-        <v>Nasa bhai</v>
+        <v/>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="str">
-        <v>1778659312652_698</v>
+        <v>1778659312652_69</v>
       </c>
       <c r="B280" t="str">
-        <v>699</v>
+        <v>70</v>
       </c>
       <c r="C280" t="str">
-        <v>1475</v>
+        <v>931</v>
       </c>
       <c r="D280" t="str">
-        <v>Tasneem bai Yusuf bhai Rail</v>
+        <v>Arwa bai Sajjadhusain bhai Partapur</v>
       </c>
       <c r="E280" t="str">
-        <v>30366367</v>
+        <v>20318614</v>
       </c>
       <c r="F280" t="str">
-        <v>Given</v>
+        <v>Pending</v>
       </c>
       <c r="G280" t="str">
         <v/>
@@ -7570,25 +7543,34 @@
     </row>
     <row r="281">
       <c r="A281" t="str">
-        <v>1778659312652_69</v>
+        <v>1778659312652_99</v>
       </c>
       <c r="B281" t="str">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="C281" t="str">
-        <v>931</v>
+        <v>236</v>
       </c>
       <c r="D281" t="str">
-        <v>Arwa bai Sajjadhusain bhai Partapur</v>
+        <v>Batul bai Johar bhai Saroda</v>
       </c>
       <c r="E281" t="str">
-        <v>20318614</v>
+        <v>30488741</v>
       </c>
       <c r="F281" t="str">
-        <v>Pending</v>
+        <v>Given</v>
       </c>
       <c r="G281" t="str">
-        <v/>
+        <v>Ilyas</v>
+      </c>
+      <c r="H281" t="str">
+        <v>24/05/2026</v>
+      </c>
+      <c r="I281" t="str">
+        <v>Sunday</v>
+      </c>
+      <c r="J281" t="str">
+        <v>22:35:04</v>
       </c>
     </row>
     <row r="282">
@@ -15147,19 +15129,19 @@
     </row>
     <row r="585">
       <c r="A585" t="str">
-        <v>1778659312652_309</v>
+        <v>1778659312652_316</v>
       </c>
       <c r="B585" t="str">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="C585" t="str">
-        <v>1146</v>
+        <v>235</v>
       </c>
       <c r="D585" t="str">
-        <v>Ismail bhai Alihusain bhai Damdi</v>
+        <v>Jumana bai Fakhruddin bhai Tarawala</v>
       </c>
       <c r="E585" t="str">
-        <v>30366733</v>
+        <v>30367675</v>
       </c>
       <c r="F585" t="str">
         <v>Pending</v>
@@ -15170,22 +15152,22 @@
     </row>
     <row r="586">
       <c r="A586" t="str">
-        <v>1778659312652_310</v>
+        <v>1778659312652_309</v>
       </c>
       <c r="B586" t="str">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C586" t="str">
-        <v>1227</v>
+        <v>1146</v>
       </c>
       <c r="D586" t="str">
-        <v>Ismail bhai Qurbanhusain bhai Billa</v>
+        <v>Ismail bhai Alihusain bhai Damdi</v>
       </c>
       <c r="E586" t="str">
-        <v>20318051</v>
+        <v>30366733</v>
       </c>
       <c r="F586" t="str">
-        <v>Given</v>
+        <v>Pending</v>
       </c>
       <c r="G586" t="str">
         <v/>
@@ -15193,22 +15175,22 @@
     </row>
     <row r="587">
       <c r="A587" t="str">
-        <v>1778659312652_311</v>
+        <v>1778659312652_310</v>
       </c>
       <c r="B587" t="str">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C587" t="str">
-        <v>1438</v>
+        <v>1227</v>
       </c>
       <c r="D587" t="str">
-        <v>Ismail bhai Saifuddin bhai Patrawala</v>
+        <v>Ismail bhai Qurbanhusain bhai Billa</v>
       </c>
       <c r="E587" t="str">
-        <v>30904442</v>
+        <v>20318051</v>
       </c>
       <c r="F587" t="str">
-        <v>Pending</v>
+        <v>Given</v>
       </c>
       <c r="G587" t="str">
         <v/>
@@ -15216,19 +15198,19 @@
     </row>
     <row r="588">
       <c r="A588" t="str">
-        <v>1778659312652_313</v>
+        <v>1778659312652_311</v>
       </c>
       <c r="B588" t="str">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="C588" t="str">
-        <v>316</v>
+        <v>1438</v>
       </c>
       <c r="D588" t="str">
-        <v>Jamila bai Ahmedali bhai Tara</v>
+        <v>Ismail bhai Saifuddin bhai Patrawala</v>
       </c>
       <c r="E588" t="str">
-        <v>20318246</v>
+        <v>30904442</v>
       </c>
       <c r="F588" t="str">
         <v>Pending</v>
@@ -15239,19 +15221,19 @@
     </row>
     <row r="589">
       <c r="A589" t="str">
-        <v>1778659312652_314</v>
+        <v>1778659312652_313</v>
       </c>
       <c r="B589" t="str">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C589" t="str">
-        <v>494</v>
+        <v>316</v>
       </c>
       <c r="D589" t="str">
-        <v>Jamila bai Najmuddin bhai Gadhiwala</v>
+        <v>Jamila bai Ahmedali bhai Tara</v>
       </c>
       <c r="E589" t="str">
-        <v>30368526</v>
+        <v>20318246</v>
       </c>
       <c r="F589" t="str">
         <v>Pending</v>
@@ -15262,22 +15244,22 @@
     </row>
     <row r="590">
       <c r="A590" t="str">
-        <v>1778659312652_315</v>
+        <v>1778659312652_314</v>
       </c>
       <c r="B590" t="str">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C590" t="str">
-        <v>304</v>
+        <v>494</v>
       </c>
       <c r="D590" t="str">
-        <v>Jumana bai Burhanuddin bhai Gabruwala</v>
+        <v>Jamila bai Najmuddin bhai Gadhiwala</v>
       </c>
       <c r="E590" t="str">
-        <v>30366585</v>
+        <v>30368526</v>
       </c>
       <c r="F590" t="str">
-        <v>Given</v>
+        <v>Pending</v>
       </c>
       <c r="G590" t="str">
         <v/>
@@ -15285,22 +15267,22 @@
     </row>
     <row r="591">
       <c r="A591" t="str">
-        <v>1778659312652_317</v>
+        <v>1778659312652_315</v>
       </c>
       <c r="B591" t="str">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="C591" t="str">
-        <v>1181</v>
+        <v>304</v>
       </c>
       <c r="D591" t="str">
-        <v>Jumana bai Hakimuddin bhai Dhambola</v>
+        <v>Jumana bai Burhanuddin bhai Gabruwala</v>
       </c>
       <c r="E591" t="str">
-        <v>30367995</v>
+        <v>30366585</v>
       </c>
       <c r="F591" t="str">
-        <v>Pending</v>
+        <v>Given</v>
       </c>
       <c r="G591" t="str">
         <v/>
@@ -15308,19 +15290,19 @@
     </row>
     <row r="592">
       <c r="A592" t="str">
-        <v>1778659312652_318</v>
+        <v>1778659312652_317</v>
       </c>
       <c r="B592" t="str">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C592" t="str">
-        <v>196</v>
+        <v>1181</v>
       </c>
       <c r="D592" t="str">
-        <v>Jumana bai Husain bhai Badshah</v>
+        <v>Jumana bai Hakimuddin bhai Dhambola</v>
       </c>
       <c r="E592" t="str">
-        <v>30368195</v>
+        <v>30367995</v>
       </c>
       <c r="F592" t="str">
         <v>Pending</v>
@@ -15331,19 +15313,19 @@
     </row>
     <row r="593">
       <c r="A593" t="str">
-        <v>1778659312652_31</v>
+        <v>1778659312652_318</v>
       </c>
       <c r="B593" t="str">
-        <v>32</v>
+        <v>319</v>
       </c>
       <c r="C593" t="str">
-        <v/>
+        <v>196</v>
       </c>
       <c r="D593" t="str">
-        <v>Ajab bai Mulla Burhanuddin bhai Mohib</v>
+        <v>Jumana bai Husain bhai Badshah</v>
       </c>
       <c r="E593" t="str">
-        <v>30391898</v>
+        <v>30368195</v>
       </c>
       <c r="F593" t="str">
         <v>Pending</v>
@@ -15354,98 +15336,89 @@
     </row>
     <row r="594">
       <c r="A594" t="str">
-        <v>1778659312652_312</v>
+        <v>1778659312652_31</v>
       </c>
       <c r="B594" t="str">
-        <v>313</v>
+        <v>32</v>
       </c>
       <c r="C594" t="str">
-        <v>160</v>
+        <v/>
       </c>
       <c r="D594" t="str">
-        <v>Jamila bai Abdullah bhai Patwari</v>
+        <v>Ajab bai Mulla Burhanuddin bhai Mohib</v>
       </c>
       <c r="E594" t="str">
-        <v>30366400</v>
+        <v>30391898</v>
       </c>
       <c r="F594" t="str">
-        <v>Given</v>
+        <v>Pending</v>
       </c>
       <c r="G594" t="str">
         <v/>
-      </c>
-      <c r="H594" t="str">
-        <v>21/05/2026</v>
-      </c>
-      <c r="I594" t="str">
-        <v>Thursday</v>
-      </c>
-      <c r="J594" t="str">
-        <v>11:02:18</v>
       </c>
     </row>
     <row r="595">
       <c r="A595" t="str">
-        <v>1778659312652_30</v>
+        <v>1778659312652_312</v>
       </c>
       <c r="B595" t="str">
-        <v>31</v>
+        <v>313</v>
       </c>
       <c r="C595" t="str">
-        <v>101</v>
+        <v>160</v>
       </c>
       <c r="D595" t="str">
-        <v>Ajab bai Mufaddal bhai Bangali</v>
+        <v>Jamila bai Abdullah bhai Patwari</v>
       </c>
       <c r="E595" t="str">
-        <v>30368206</v>
+        <v>30366400</v>
       </c>
       <c r="F595" t="str">
         <v>Given</v>
       </c>
       <c r="G595" t="str">
-        <v>Insiya ben pachlasa</v>
+        <v/>
       </c>
       <c r="H595" t="str">
-        <v>23/05/2026</v>
+        <v>21/05/2026</v>
       </c>
       <c r="I595" t="str">
-        <v>Saturday</v>
+        <v>Thursday</v>
       </c>
       <c r="J595" t="str">
-        <v>12:14:22</v>
+        <v>11:02:18</v>
       </c>
     </row>
     <row r="596">
       <c r="A596" t="str">
-        <v>1778659312652_316</v>
+        <v>1778659312652_30</v>
       </c>
       <c r="B596" t="str">
-        <v>317</v>
+        <v>31</v>
       </c>
       <c r="C596" t="str">
-        <v>235</v>
+        <v>101</v>
       </c>
       <c r="D596" t="str">
-        <v>Jumana bai Fakhruddin bhai Tarawala</v>
+        <v>Ajab bai Mufaddal bhai Bangali</v>
       </c>
       <c r="E596" t="str">
-        <v>30367675</v>
+        <v>30368206</v>
       </c>
       <c r="F596" t="str">
         <v>Given</v>
       </c>
       <c r="G596" t="str">
-        <v>Ilyas</v>
+        <v>Insiya ben pachlasa</v>
       </c>
       <c r="H596" t="str">
-        <v>24/05/2026</v>
+        <v>23/05/2026</v>
       </c>
       <c r="I596" t="str">
-        <v>Sunday</v>
+        <v>Saturday</v>
       </c>
       <c r="J596" t="str">
-        <v>20:53:42</v>
+        <v>12:14:22</v>
       </c>
     </row>
     <row r="597">

</xml_diff>

<commit_message>
ACC NO first prefrence for search
</commit_message>
<xml_diff>
--- a/backend/distribution_live_backup.xlsx
+++ b/backend/distribution_live_backup.xlsx
@@ -6969,77 +6969,77 @@
     </row>
     <row r="258">
       <c r="A258" t="str">
-        <v>1778659312652_99</v>
+        <v>1778659312652_100</v>
       </c>
       <c r="B258" t="str">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C258" t="str">
-        <v>236</v>
+        <v>117</v>
       </c>
       <c r="D258" t="str">
-        <v>Batul bai Johar bhai Saroda</v>
+        <v>Batul bai Mohammadhussain bhai Bankoda</v>
       </c>
       <c r="E258" t="str">
-        <v>30488741</v>
+        <v>30360295</v>
       </c>
       <c r="F258" t="str">
-        <v>Pending</v>
+        <v>Given</v>
       </c>
       <c r="G258" t="str">
         <v/>
+      </c>
+      <c r="H258" t="str">
+        <v>22/05/2026</v>
+      </c>
+      <c r="I258" t="str">
+        <v>Friday</v>
+      </c>
+      <c r="J258" t="str">
+        <v>12:19:42</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="str">
-        <v>1778659312652_100</v>
+        <v>1778659312652_101</v>
       </c>
       <c r="B259" t="str">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C259" t="str">
-        <v>117</v>
+        <v>254</v>
       </c>
       <c r="D259" t="str">
-        <v>Batul bai Mohammadhussain bhai Bankoda</v>
+        <v>Batul bai Mohammadhussain bhai Patra</v>
       </c>
       <c r="E259" t="str">
-        <v>30360295</v>
+        <v>20318132</v>
       </c>
       <c r="F259" t="str">
-        <v>Given</v>
+        <v>Pending</v>
       </c>
       <c r="G259" t="str">
         <v/>
-      </c>
-      <c r="H259" t="str">
-        <v>22/05/2026</v>
-      </c>
-      <c r="I259" t="str">
-        <v>Friday</v>
-      </c>
-      <c r="J259" t="str">
-        <v>12:19:42</v>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="str">
-        <v>1778659312652_101</v>
+        <v>1778659312652_99</v>
       </c>
       <c r="B260" t="str">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C260" t="str">
-        <v>254</v>
+        <v>236</v>
       </c>
       <c r="D260" t="str">
-        <v>Batul bai Mohammadhussain bhai Patra</v>
+        <v>Batul bai Johar bhai Saroda</v>
       </c>
       <c r="E260" t="str">
-        <v>20318132</v>
+        <v>30488741</v>
       </c>
       <c r="F260" t="str">
-        <v>Pending</v>
+        <v>Given</v>
       </c>
       <c r="G260" t="str">
         <v/>
@@ -15189,19 +15189,19 @@
     </row>
     <row r="588">
       <c r="A588" t="str">
-        <v>1778659312652_316</v>
+        <v>1778659312652_313</v>
       </c>
       <c r="B588" t="str">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="C588" t="str">
-        <v>235</v>
+        <v>316</v>
       </c>
       <c r="D588" t="str">
-        <v>Jumana bai Fakhruddin bhai Tarawala</v>
+        <v>Jamila bai Ahmedali bhai Tara</v>
       </c>
       <c r="E588" t="str">
-        <v>30367675</v>
+        <v>20318246</v>
       </c>
       <c r="F588" t="str">
         <v>Pending</v>
@@ -15212,19 +15212,19 @@
     </row>
     <row r="589">
       <c r="A589" t="str">
-        <v>1778659312652_313</v>
+        <v>1778659312652_314</v>
       </c>
       <c r="B589" t="str">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C589" t="str">
-        <v>316</v>
+        <v>494</v>
       </c>
       <c r="D589" t="str">
-        <v>Jamila bai Ahmedali bhai Tara</v>
+        <v>Jamila bai Najmuddin bhai Gadhiwala</v>
       </c>
       <c r="E589" t="str">
-        <v>20318246</v>
+        <v>30368526</v>
       </c>
       <c r="F589" t="str">
         <v>Pending</v>
@@ -15235,22 +15235,22 @@
     </row>
     <row r="590">
       <c r="A590" t="str">
-        <v>1778659312652_314</v>
+        <v>1778659312652_315</v>
       </c>
       <c r="B590" t="str">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C590" t="str">
-        <v>494</v>
+        <v>304</v>
       </c>
       <c r="D590" t="str">
-        <v>Jamila bai Najmuddin bhai Gadhiwala</v>
+        <v>Jumana bai Burhanuddin bhai Gabruwala</v>
       </c>
       <c r="E590" t="str">
-        <v>30368526</v>
+        <v>30366585</v>
       </c>
       <c r="F590" t="str">
-        <v>Pending</v>
+        <v>Given</v>
       </c>
       <c r="G590" t="str">
         <v/>
@@ -15258,22 +15258,22 @@
     </row>
     <row r="591">
       <c r="A591" t="str">
-        <v>1778659312652_315</v>
+        <v>1778659312652_317</v>
       </c>
       <c r="B591" t="str">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="C591" t="str">
-        <v>304</v>
+        <v>1181</v>
       </c>
       <c r="D591" t="str">
-        <v>Jumana bai Burhanuddin bhai Gabruwala</v>
+        <v>Jumana bai Hakimuddin bhai Dhambola</v>
       </c>
       <c r="E591" t="str">
-        <v>30366585</v>
+        <v>30367995</v>
       </c>
       <c r="F591" t="str">
-        <v>Given</v>
+        <v>Pending</v>
       </c>
       <c r="G591" t="str">
         <v/>
@@ -15281,19 +15281,19 @@
     </row>
     <row r="592">
       <c r="A592" t="str">
-        <v>1778659312652_317</v>
+        <v>1778659312652_318</v>
       </c>
       <c r="B592" t="str">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C592" t="str">
-        <v>1181</v>
+        <v>196</v>
       </c>
       <c r="D592" t="str">
-        <v>Jumana bai Hakimuddin bhai Dhambola</v>
+        <v>Jumana bai Husain bhai Badshah</v>
       </c>
       <c r="E592" t="str">
-        <v>30367995</v>
+        <v>30368195</v>
       </c>
       <c r="F592" t="str">
         <v>Pending</v>
@@ -15304,19 +15304,19 @@
     </row>
     <row r="593">
       <c r="A593" t="str">
-        <v>1778659312652_318</v>
+        <v>1778659312652_31</v>
       </c>
       <c r="B593" t="str">
-        <v>319</v>
+        <v>32</v>
       </c>
       <c r="C593" t="str">
-        <v>196</v>
+        <v/>
       </c>
       <c r="D593" t="str">
-        <v>Jumana bai Husain bhai Badshah</v>
+        <v>Ajab bai Mulla Burhanuddin bhai Mohib</v>
       </c>
       <c r="E593" t="str">
-        <v>30368195</v>
+        <v>30391898</v>
       </c>
       <c r="F593" t="str">
         <v>Pending</v>
@@ -15327,57 +15327,57 @@
     </row>
     <row r="594">
       <c r="A594" t="str">
-        <v>1778659312652_31</v>
+        <v>1778659312652_312</v>
       </c>
       <c r="B594" t="str">
-        <v>32</v>
+        <v>313</v>
       </c>
       <c r="C594" t="str">
-        <v/>
+        <v>160</v>
       </c>
       <c r="D594" t="str">
-        <v>Ajab bai Mulla Burhanuddin bhai Mohib</v>
+        <v>Jamila bai Abdullah bhai Patwari</v>
       </c>
       <c r="E594" t="str">
-        <v>30391898</v>
+        <v>30366400</v>
       </c>
       <c r="F594" t="str">
-        <v>Pending</v>
+        <v>Given</v>
       </c>
       <c r="G594" t="str">
         <v/>
+      </c>
+      <c r="H594" t="str">
+        <v>21/05/2026</v>
+      </c>
+      <c r="I594" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="J594" t="str">
+        <v>11:02:18</v>
       </c>
     </row>
     <row r="595">
       <c r="A595" t="str">
-        <v>1778659312652_312</v>
+        <v>1778659312652_316</v>
       </c>
       <c r="B595" t="str">
-        <v>313</v>
+        <v>317</v>
       </c>
       <c r="C595" t="str">
-        <v>160</v>
+        <v>235</v>
       </c>
       <c r="D595" t="str">
-        <v>Jamila bai Abdullah bhai Patwari</v>
+        <v>Jumana bai Fakhruddin bhai Tarawala</v>
       </c>
       <c r="E595" t="str">
-        <v>30366400</v>
+        <v>30367675</v>
       </c>
       <c r="F595" t="str">
-        <v>Given</v>
+        <v>Pending</v>
       </c>
       <c r="G595" t="str">
         <v/>
-      </c>
-      <c r="H595" t="str">
-        <v>21/05/2026</v>
-      </c>
-      <c r="I595" t="str">
-        <v>Thursday</v>
-      </c>
-      <c r="J595" t="str">
-        <v>11:02:18</v>
       </c>
     </row>
     <row r="596">

</xml_diff>

<commit_message>
bulk distribution design change
</commit_message>
<xml_diff>
--- a/backend/distribution_live_backup.xlsx
+++ b/backend/distribution_live_backup.xlsx
@@ -7059,74 +7059,83 @@
     </row>
     <row r="258">
       <c r="A258" t="str">
-        <v>1778659312652_100</v>
+        <v>1778659312652_99</v>
       </c>
       <c r="B258" t="str">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C258" t="str">
-        <v>117</v>
+        <v>236</v>
       </c>
       <c r="D258" t="str">
-        <v>Batul bai Mohammadhussain bhai Bankoda</v>
+        <v>Batul bai Johar bhai Saroda</v>
       </c>
       <c r="E258" t="str">
-        <v>30360295</v>
+        <v>30488741</v>
       </c>
       <c r="F258" t="str">
         <v>Given</v>
       </c>
       <c r="G258" t="str">
-        <v/>
+        <v>Ilyas</v>
       </c>
       <c r="H258" t="str">
-        <v>22/05/2026</v>
+        <v>25/05/2026</v>
       </c>
       <c r="I258" t="str">
-        <v>Friday</v>
+        <v>Monday</v>
       </c>
       <c r="J258" t="str">
-        <v>12:19:42</v>
+        <v>16:05:11</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="str">
-        <v>1778659312652_101</v>
+        <v>1778659312652_100</v>
       </c>
       <c r="B259" t="str">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C259" t="str">
-        <v>254</v>
+        <v>117</v>
       </c>
       <c r="D259" t="str">
-        <v>Batul bai Mohammadhussain bhai Patra</v>
+        <v>Batul bai Mohammadhussain bhai Bankoda</v>
       </c>
       <c r="E259" t="str">
-        <v>20318132</v>
+        <v>30360295</v>
       </c>
       <c r="F259" t="str">
-        <v>Pending</v>
+        <v>Given</v>
       </c>
       <c r="G259" t="str">
         <v/>
+      </c>
+      <c r="H259" t="str">
+        <v>22/05/2026</v>
+      </c>
+      <c r="I259" t="str">
+        <v>Friday</v>
+      </c>
+      <c r="J259" t="str">
+        <v>12:19:42</v>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="str">
-        <v>1778659312652_103</v>
+        <v>1778659312652_101</v>
       </c>
       <c r="B260" t="str">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C260" t="str">
-        <v>1303</v>
+        <v>254</v>
       </c>
       <c r="D260" t="str">
-        <v>Batul bai Qutbuddin bhai Rustam</v>
+        <v>Batul bai Mohammadhussain bhai Patra</v>
       </c>
       <c r="E260" t="str">
-        <v>30366656</v>
+        <v>20318132</v>
       </c>
       <c r="F260" t="str">
         <v>Pending</v>
@@ -7137,19 +7146,19 @@
     </row>
     <row r="261">
       <c r="A261" t="str">
-        <v>1778659312652_104</v>
+        <v>1778659312652_103</v>
       </c>
       <c r="B261" t="str">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C261" t="str">
-        <v>76</v>
+        <v>1303</v>
       </c>
       <c r="D261" t="str">
-        <v>Batul bai Saifuddin bhai Doodhbhai</v>
+        <v>Batul bai Qutbuddin bhai Rustam</v>
       </c>
       <c r="E261" t="str">
-        <v>30368616</v>
+        <v>30366656</v>
       </c>
       <c r="F261" t="str">
         <v>Pending</v>
@@ -7160,19 +7169,19 @@
     </row>
     <row r="262">
       <c r="A262" t="str">
-        <v>1778659312652_105</v>
+        <v>1778659312652_104</v>
       </c>
       <c r="B262" t="str">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C262" t="str">
-        <v>744</v>
+        <v>76</v>
       </c>
       <c r="D262" t="str">
-        <v>Batul bai Shaikh Akbarhusain bhai Rampurwala</v>
+        <v>Batul bai Saifuddin bhai Doodhbhai</v>
       </c>
       <c r="E262" t="str">
-        <v>30367359</v>
+        <v>30368616</v>
       </c>
       <c r="F262" t="str">
         <v>Pending</v>
@@ -7183,89 +7192,80 @@
     </row>
     <row r="263">
       <c r="A263" t="str">
-        <v>1778659312652_106</v>
+        <v>1778659312652_105</v>
       </c>
       <c r="B263" t="str">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C263" t="str">
-        <v>807</v>
+        <v>744</v>
       </c>
       <c r="D263" t="str">
-        <v>Batul bai Taiyebali bhai Bankoda</v>
+        <v>Batul bai Shaikh Akbarhusain bhai Rampurwala</v>
       </c>
       <c r="E263" t="str">
-        <v>30367508</v>
+        <v>30367359</v>
       </c>
       <c r="F263" t="str">
-        <v>Given</v>
+        <v>Pending</v>
       </c>
       <c r="G263" t="str">
-        <v>zainab ben antri</v>
-      </c>
-      <c r="H263" t="str">
-        <v>18/05/2026</v>
-      </c>
-      <c r="I263" t="str">
-        <v>Monday</v>
-      </c>
-      <c r="J263" t="str">
-        <v>11:50:34</v>
+        <v/>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="str">
-        <v>1778659312652_6</v>
+        <v>1778659312652_106</v>
       </c>
       <c r="B264" t="str">
-        <v>7</v>
+        <v>107</v>
       </c>
       <c r="C264" t="str">
-        <v>7</v>
+        <v>807</v>
       </c>
       <c r="D264" t="str">
-        <v>Abbas bhai Alihusain bhai Sihjee</v>
+        <v>Batul bai Taiyebali bhai Bankoda</v>
       </c>
       <c r="E264" t="str">
-        <v>20435003</v>
+        <v>30367508</v>
       </c>
       <c r="F264" t="str">
         <v>Given</v>
       </c>
       <c r="G264" t="str">
-        <v>Ajab ben Khand</v>
+        <v>zainab ben antri</v>
       </c>
       <c r="H264" t="str">
-        <v>21/05/2026</v>
+        <v>18/05/2026</v>
       </c>
       <c r="I264" t="str">
-        <v>Thursday</v>
+        <v>Monday</v>
       </c>
       <c r="J264" t="str">
-        <v>10:25:43</v>
+        <v>11:50:34</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="str">
-        <v>1778659312652_335</v>
+        <v>1778659312652_6</v>
       </c>
       <c r="B265" t="str">
-        <v>336</v>
+        <v>7</v>
       </c>
       <c r="C265" t="str">
-        <v>1197</v>
+        <v>7</v>
       </c>
       <c r="D265" t="str">
-        <v>Khanali bhai Mohammadhussain bhai Hedari</v>
+        <v>Abbas bhai Alihusain bhai Sihjee</v>
       </c>
       <c r="E265" t="str">
-        <v>20414120</v>
+        <v>20435003</v>
       </c>
       <c r="F265" t="str">
         <v>Given</v>
       </c>
       <c r="G265" t="str">
-        <v/>
+        <v>Ajab ben Khand</v>
       </c>
       <c r="H265" t="str">
         <v>21/05/2026</v>
@@ -7274,47 +7274,56 @@
         <v>Thursday</v>
       </c>
       <c r="J265" t="str">
-        <v>11:08:30</v>
+        <v>10:25:43</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="str">
-        <v>1778659312652_108</v>
+        <v>1778659312652_335</v>
       </c>
       <c r="B266" t="str">
-        <v>109</v>
+        <v>336</v>
       </c>
       <c r="C266" t="str">
-        <v>588</v>
+        <v>1197</v>
       </c>
       <c r="D266" t="str">
-        <v>Bilqis bai Husain bhai Gadi</v>
+        <v>Khanali bhai Mohammadhussain bhai Hedari</v>
       </c>
       <c r="E266" t="str">
-        <v>20318760</v>
+        <v>20414120</v>
       </c>
       <c r="F266" t="str">
-        <v>Pending</v>
+        <v>Given</v>
       </c>
       <c r="G266" t="str">
         <v/>
+      </c>
+      <c r="H266" t="str">
+        <v>21/05/2026</v>
+      </c>
+      <c r="I266" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="J266" t="str">
+        <v>11:08:30</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="str">
-        <v>1778659312652_326</v>
+        <v>1778659312652_108</v>
       </c>
       <c r="B267" t="str">
-        <v>327</v>
+        <v>109</v>
       </c>
       <c r="C267" t="str">
-        <v>431</v>
+        <v>588</v>
       </c>
       <c r="D267" t="str">
-        <v>Khadija bai Fakhruddin bhai Peeth</v>
+        <v>Bilqis bai Husain bhai Gadi</v>
       </c>
       <c r="E267" t="str">
-        <v>30366840</v>
+        <v>20318760</v>
       </c>
       <c r="F267" t="str">
         <v>Pending</v>
@@ -7325,19 +7334,19 @@
     </row>
     <row r="268">
       <c r="A268" t="str">
-        <v>1778659312652_327</v>
+        <v>1778659312652_326</v>
       </c>
       <c r="B268" t="str">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C268" t="str">
-        <v>822</v>
+        <v>431</v>
       </c>
       <c r="D268" t="str">
-        <v>Khadija bai Ghulamhusain bhai Dudhwala</v>
+        <v>Khadija bai Fakhruddin bhai Peeth</v>
       </c>
       <c r="E268" t="str">
-        <v>30367535</v>
+        <v>30366840</v>
       </c>
       <c r="F268" t="str">
         <v>Pending</v>
@@ -7348,19 +7357,19 @@
     </row>
     <row r="269">
       <c r="A269" t="str">
-        <v>1778659312652_328</v>
+        <v>1778659312652_327</v>
       </c>
       <c r="B269" t="str">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C269" t="str">
-        <v>684</v>
+        <v>822</v>
       </c>
       <c r="D269" t="str">
-        <v>Khadija bai Haiderali bhai Maudi wala</v>
+        <v>Khadija bai Ghulamhusain bhai Dudhwala</v>
       </c>
       <c r="E269" t="str">
-        <v>30367251</v>
+        <v>30367535</v>
       </c>
       <c r="F269" t="str">
         <v>Pending</v>
@@ -7371,97 +7380,97 @@
     </row>
     <row r="270">
       <c r="A270" t="str">
-        <v>1778659312652_102</v>
+        <v>1778659312652_328</v>
       </c>
       <c r="B270" t="str">
-        <v>103</v>
+        <v>329</v>
       </c>
       <c r="C270" t="str">
-        <v>637</v>
+        <v>684</v>
       </c>
       <c r="D270" t="str">
-        <v>Batul bai Mufaddal bhai Jaan</v>
+        <v>Khadija bai Haiderali bhai Maudi wala</v>
       </c>
       <c r="E270" t="str">
-        <v>30367654</v>
+        <v>30367251</v>
       </c>
       <c r="F270" t="str">
-        <v>Given</v>
+        <v>Pending</v>
       </c>
       <c r="G270" t="str">
-        <v>mulla jivaji</v>
-      </c>
-      <c r="H270" t="str">
-        <v>22/05/2026</v>
-      </c>
-      <c r="I270" t="str">
-        <v>Friday</v>
-      </c>
-      <c r="J270" t="str">
-        <v>11:47:31</v>
+        <v/>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="str">
-        <v>1778659312652_330</v>
+        <v>1778659312652_102</v>
       </c>
       <c r="B271" t="str">
-        <v>331</v>
+        <v>103</v>
       </c>
       <c r="C271" t="str">
-        <v>1356</v>
+        <v>637</v>
       </c>
       <c r="D271" t="str">
-        <v>Khadija bai Murtaza bhai Ratawala</v>
+        <v>Batul bai Mufaddal bhai Jaan</v>
       </c>
       <c r="E271" t="str">
-        <v>30367899</v>
+        <v>30367654</v>
       </c>
       <c r="F271" t="str">
         <v>Given</v>
       </c>
       <c r="G271" t="str">
-        <v>Fakhruddin kawja</v>
+        <v>mulla jivaji</v>
+      </c>
+      <c r="H271" t="str">
+        <v>22/05/2026</v>
+      </c>
+      <c r="I271" t="str">
+        <v>Friday</v>
+      </c>
+      <c r="J271" t="str">
+        <v>11:47:31</v>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="str">
-        <v>1778659312652_331</v>
+        <v>1778659312652_330</v>
       </c>
       <c r="B272" t="str">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C272" t="str">
-        <v>388</v>
+        <v>1356</v>
       </c>
       <c r="D272" t="str">
-        <v>Khadija bai Qutbuddin bhai Tara</v>
+        <v>Khadija bai Murtaza bhai Ratawala</v>
       </c>
       <c r="E272" t="str">
-        <v>30366583</v>
+        <v>30367899</v>
       </c>
       <c r="F272" t="str">
-        <v>Pending</v>
+        <v>Given</v>
       </c>
       <c r="G272" t="str">
-        <v/>
+        <v>Fakhruddin kawja</v>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="str">
-        <v>1778659312652_332</v>
+        <v>1778659312652_331</v>
       </c>
       <c r="B273" t="str">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C273" t="str">
-        <v>310</v>
+        <v>388</v>
       </c>
       <c r="D273" t="str">
-        <v>Khadija bai Saifuddin bhai Ezzi</v>
+        <v>Khadija bai Qutbuddin bhai Tara</v>
       </c>
       <c r="E273" t="str">
-        <v>30366643</v>
+        <v>30366583</v>
       </c>
       <c r="F273" t="str">
         <v>Pending</v>
@@ -7472,80 +7481,71 @@
     </row>
     <row r="274">
       <c r="A274" t="str">
-        <v>1778659312652_333</v>
+        <v>1778659312652_332</v>
       </c>
       <c r="B274" t="str">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C274" t="str">
-        <v>1029</v>
+        <v>310</v>
       </c>
       <c r="D274" t="str">
-        <v>Khadija bai Shaikh Mohammed bhai Khumanpur</v>
+        <v>Khadija bai Saifuddin bhai Ezzi</v>
       </c>
       <c r="E274" t="str">
-        <v>30367849</v>
+        <v>30366643</v>
       </c>
       <c r="F274" t="str">
-        <v>Given</v>
+        <v>Pending</v>
       </c>
       <c r="G274" t="str">
-        <v>yakut bhai gaba</v>
+        <v/>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="str">
-        <v>1778659312652_334</v>
+        <v>1778659312652_333</v>
       </c>
       <c r="B275" t="str">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C275" t="str">
-        <v>138</v>
+        <v>1029</v>
       </c>
       <c r="D275" t="str">
-        <v>Khadija bai Tayyeb bhai Gadi</v>
+        <v>Khadija bai Shaikh Mohammed bhai Khumanpur</v>
       </c>
       <c r="E275" t="str">
-        <v>30366336</v>
+        <v>30367849</v>
       </c>
       <c r="F275" t="str">
         <v>Given</v>
       </c>
       <c r="G275" t="str">
-        <v>shkh fakhruddin badi</v>
+        <v>yakut bhai gaba</v>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="str">
-        <v>1778659312652_99</v>
+        <v>1778659312652_334</v>
       </c>
       <c r="B276" t="str">
-        <v>100</v>
+        <v>335</v>
       </c>
       <c r="C276" t="str">
-        <v>236</v>
+        <v>138</v>
       </c>
       <c r="D276" t="str">
-        <v>Batul bai Johar bhai Saroda</v>
+        <v>Khadija bai Tayyeb bhai Gadi</v>
       </c>
       <c r="E276" t="str">
-        <v>30488741</v>
+        <v>30366336</v>
       </c>
       <c r="F276" t="str">
         <v>Given</v>
       </c>
       <c r="G276" t="str">
-        <v>Ilyas</v>
-      </c>
-      <c r="H276" t="str">
-        <v>25/05/2026</v>
-      </c>
-      <c r="I276" t="str">
-        <v>Monday</v>
-      </c>
-      <c r="J276" t="str">
-        <v>03:34:44</v>
+        <v>shkh fakhruddin badi</v>
       </c>
     </row>
     <row r="277">
@@ -15601,66 +15601,57 @@
     </row>
     <row r="593">
       <c r="A593" t="str">
-        <v>1778659312652_30</v>
+        <v>1778659312652_316</v>
       </c>
       <c r="B593" t="str">
-        <v>31</v>
+        <v>317</v>
       </c>
       <c r="C593" t="str">
-        <v>101</v>
+        <v>235</v>
       </c>
       <c r="D593" t="str">
-        <v>Ajab bai Mufaddal bhai Bangali</v>
+        <v>Jumana bai Fakhruddin bhai Tarawala</v>
       </c>
       <c r="E593" t="str">
-        <v>30368206</v>
+        <v>30367675</v>
       </c>
       <c r="F593" t="str">
-        <v>Given</v>
+        <v>Pending</v>
       </c>
       <c r="G593" t="str">
-        <v>Insiya ben pachlasa</v>
-      </c>
-      <c r="H593" t="str">
-        <v>23/05/2026</v>
-      </c>
-      <c r="I593" t="str">
-        <v>Saturday</v>
-      </c>
-      <c r="J593" t="str">
-        <v>12:14:22</v>
+        <v/>
       </c>
     </row>
     <row r="594">
       <c r="A594" t="str">
-        <v>1778659312652_316</v>
+        <v>1778659312652_30</v>
       </c>
       <c r="B594" t="str">
-        <v>317</v>
+        <v>31</v>
       </c>
       <c r="C594" t="str">
-        <v>235</v>
+        <v>101</v>
       </c>
       <c r="D594" t="str">
-        <v>Jumana bai Fakhruddin bhai Tarawala</v>
+        <v>Ajab bai Mufaddal bhai Bangali</v>
       </c>
       <c r="E594" t="str">
-        <v>30367675</v>
+        <v>30368206</v>
       </c>
       <c r="F594" t="str">
-        <v>Pending</v>
+        <v>Given</v>
       </c>
       <c r="G594" t="str">
-        <v/>
+        <v>Insiya ben pachlasa</v>
       </c>
       <c r="H594" t="str">
-        <v>25/05/2026</v>
+        <v>23/05/2026</v>
       </c>
       <c r="I594" t="str">
-        <v>Monday</v>
+        <v>Saturday</v>
       </c>
       <c r="J594" t="str">
-        <v>03:35:08</v>
+        <v>12:14:22</v>
       </c>
     </row>
     <row r="595">

</xml_diff>

<commit_message>
DistributionTable filter design change
</commit_message>
<xml_diff>
--- a/backend/distribution_live_backup.xlsx
+++ b/backend/distribution_live_backup.xlsx
@@ -7059,66 +7059,57 @@
     </row>
     <row r="258">
       <c r="A258" t="str">
-        <v>1778659312652_99</v>
+        <v>1778659312652_100</v>
       </c>
       <c r="B258" t="str">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C258" t="str">
-        <v>236</v>
+        <v>117</v>
       </c>
       <c r="D258" t="str">
-        <v>Batul bai Johar bhai Saroda</v>
+        <v>Batul bai Mohammadhussain bhai Bankoda</v>
       </c>
       <c r="E258" t="str">
-        <v>30488741</v>
+        <v>30360295</v>
       </c>
       <c r="F258" t="str">
         <v>Given</v>
       </c>
       <c r="G258" t="str">
-        <v>Ilyas</v>
+        <v/>
       </c>
       <c r="H258" t="str">
-        <v>25/05/2026</v>
+        <v>22/05/2026</v>
       </c>
       <c r="I258" t="str">
-        <v>Monday</v>
+        <v>Friday</v>
       </c>
       <c r="J258" t="str">
-        <v>16:05:11</v>
+        <v>12:19:42</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="str">
-        <v>1778659312652_100</v>
+        <v>1778659312652_99</v>
       </c>
       <c r="B259" t="str">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C259" t="str">
-        <v>117</v>
+        <v>236</v>
       </c>
       <c r="D259" t="str">
-        <v>Batul bai Mohammadhussain bhai Bankoda</v>
+        <v>Batul bai Johar bhai Saroda</v>
       </c>
       <c r="E259" t="str">
-        <v>30360295</v>
+        <v>30488741</v>
       </c>
       <c r="F259" t="str">
         <v>Given</v>
       </c>
       <c r="G259" t="str">
-        <v/>
-      </c>
-      <c r="H259" t="str">
-        <v>22/05/2026</v>
-      </c>
-      <c r="I259" t="str">
-        <v>Friday</v>
-      </c>
-      <c r="J259" t="str">
-        <v>12:19:42</v>
+        <v>Ilyas</v>
       </c>
     </row>
     <row r="260">

</xml_diff>

<commit_message>
feat: optimize bulk verification UI with virtual scroll, interactive filters, and inline actions
</commit_message>
<xml_diff>
--- a/backend/distribution_live_backup.xlsx
+++ b/backend/distribution_live_backup.xlsx
@@ -15183,97 +15183,106 @@
     </row>
     <row r="576">
       <c r="A576" t="str">
-        <v>1778659312652_603</v>
+        <v>1778659312652_592</v>
       </c>
       <c r="B576" t="str">
-        <v>604</v>
+        <v>593</v>
       </c>
       <c r="C576" t="str">
-        <v>323</v>
+        <v>380</v>
       </c>
       <c r="D576" t="str">
-        <v>Shaikh Asgarali bhai Ahmedali bhai Khajoori</v>
+        <v>Shabbirhusain bhai Qurbanhusain bhai Thakerdawala</v>
       </c>
       <c r="E576" t="str">
-        <v>20352038</v>
+        <v>20436086</v>
       </c>
       <c r="F576" t="str">
-        <v>Not Allowed</v>
+        <v>Given</v>
       </c>
       <c r="G576" t="str">
         <v/>
+      </c>
+      <c r="H576" t="str">
+        <v>23/05/2026</v>
+      </c>
+      <c r="I576" t="str">
+        <v>Saturday</v>
+      </c>
+      <c r="J576" t="str">
+        <v>11:07:15</v>
       </c>
     </row>
     <row r="577">
       <c r="A577" t="str">
-        <v>1778659312652_592</v>
+        <v>1778659312652_603</v>
       </c>
       <c r="B577" t="str">
-        <v>593</v>
+        <v>604</v>
       </c>
       <c r="C577" t="str">
-        <v>380</v>
+        <v>323</v>
       </c>
       <c r="D577" t="str">
-        <v>Shabbirhusain bhai Qurbanhusain bhai Thakerdawala</v>
+        <v>Shaikh Asgarali bhai Ahmedali bhai Khajoori</v>
       </c>
       <c r="E577" t="str">
-        <v>20436086</v>
+        <v>20352038</v>
       </c>
       <c r="F577" t="str">
-        <v>Given</v>
+        <v>Not Allowed</v>
       </c>
       <c r="G577" t="str">
         <v/>
-      </c>
-      <c r="H577" t="str">
-        <v>23/05/2026</v>
-      </c>
-      <c r="I577" t="str">
-        <v>Saturday</v>
-      </c>
-      <c r="J577" t="str">
-        <v>11:07:15</v>
       </c>
     </row>
     <row r="578">
       <c r="A578" t="str">
-        <v>1778659312652_586</v>
+        <v>1778659312652_596</v>
       </c>
       <c r="B578" t="str">
-        <v>587</v>
+        <v>597</v>
       </c>
       <c r="C578" t="str">
-        <v>1476</v>
+        <v>70</v>
       </c>
       <c r="D578" t="str">
-        <v>Shabbir bhai Taiyebali bhai Sukhsar</v>
+        <v>Shaikh Abbas bhai Mulla Baqir bhai Damriwala</v>
       </c>
       <c r="E578" t="str">
-        <v>20406259</v>
+        <v>20407514</v>
       </c>
       <c r="F578" t="str">
-        <v>Pending</v>
+        <v>Given</v>
       </c>
       <c r="G578" t="str">
-        <v/>
+        <v>Hakimuddin bhai popat</v>
+      </c>
+      <c r="H578" t="str">
+        <v>28/05/2026</v>
+      </c>
+      <c r="I578" t="str">
+        <v>Thursday</v>
+      </c>
+      <c r="J578" t="str">
+        <v>11:55:25</v>
       </c>
     </row>
     <row r="579">
       <c r="A579" t="str">
-        <v>1778659312652_591</v>
+        <v>1778659312652_586</v>
       </c>
       <c r="B579" t="str">
-        <v>592</v>
+        <v>587</v>
       </c>
       <c r="C579" t="str">
-        <v>54</v>
+        <v>1476</v>
       </c>
       <c r="D579" t="str">
-        <v>Shabbirhusain bhai Qurbanhusain bhai Pachlasa</v>
+        <v>Shabbir bhai Taiyebali bhai Sukhsar</v>
       </c>
       <c r="E579" t="str">
-        <v>20402355</v>
+        <v>20406259</v>
       </c>
       <c r="F579" t="str">
         <v>Pending</v>
@@ -15284,19 +15293,19 @@
     </row>
     <row r="580">
       <c r="A580" t="str">
-        <v>1778659312652_593</v>
+        <v>1778659312652_591</v>
       </c>
       <c r="B580" t="str">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="C580" t="str">
-        <v>472</v>
+        <v>54</v>
       </c>
       <c r="D580" t="str">
-        <v>Shabbirhusain bhai Taherali bhai Munshi</v>
+        <v>Shabbirhusain bhai Qurbanhusain bhai Pachlasa</v>
       </c>
       <c r="E580" t="str">
-        <v>20318697</v>
+        <v>20402355</v>
       </c>
       <c r="F580" t="str">
         <v>Pending</v>
@@ -15307,19 +15316,19 @@
     </row>
     <row r="581">
       <c r="A581" t="str">
-        <v>1778659312652_594</v>
+        <v>1778659312652_593</v>
       </c>
       <c r="B581" t="str">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="C581" t="str">
-        <v>1111</v>
+        <v>472</v>
       </c>
       <c r="D581" t="str">
-        <v>Shaikh Abbas bhai Ali bhai Kika bhai</v>
+        <v>Shabbirhusain bhai Taherali bhai Munshi</v>
       </c>
       <c r="E581" t="str">
-        <v>20387729</v>
+        <v>20318697</v>
       </c>
       <c r="F581" t="str">
         <v>Pending</v>
@@ -15330,19 +15339,19 @@
     </row>
     <row r="582">
       <c r="A582" t="str">
-        <v>1778659312652_595</v>
+        <v>1778659312652_594</v>
       </c>
       <c r="B582" t="str">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="C582" t="str">
-        <v>1260</v>
+        <v>1111</v>
       </c>
       <c r="D582" t="str">
-        <v>Shaikh Abbas bhai Mohammadhussain bhai Jamali</v>
+        <v>Shaikh Abbas bhai Ali bhai Kika bhai</v>
       </c>
       <c r="E582" t="str">
-        <v>20352092</v>
+        <v>20387729</v>
       </c>
       <c r="F582" t="str">
         <v>Pending</v>
@@ -15353,22 +15362,22 @@
     </row>
     <row r="583">
       <c r="A583" t="str">
-        <v>1778659312652_596</v>
+        <v>1778659312652_595</v>
       </c>
       <c r="B583" t="str">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="C583" t="str">
-        <v>70</v>
+        <v>1260</v>
       </c>
       <c r="D583" t="str">
-        <v>Shaikh Abbas bhai Mulla Baqir bhai Damriwala</v>
+        <v>Shaikh Abbas bhai Mohammadhussain bhai Jamali</v>
       </c>
       <c r="E583" t="str">
-        <v>20407514</v>
+        <v>20352092</v>
       </c>
       <c r="F583" t="str">
-        <v>Not Allowed</v>
+        <v>Pending</v>
       </c>
       <c r="G583" t="str">
         <v/>

</xml_diff>

<commit_message>
fix frontend lag and implement data pagination
</commit_message>
<xml_diff>
--- a/backend/distribution_live_backup.xlsx
+++ b/backend/distribution_live_backup.xlsx
@@ -7091,48 +7091,48 @@
     </row>
     <row r="259">
       <c r="A259" t="str">
-        <v>1778659312652_99</v>
+        <v>1778659312652_101</v>
       </c>
       <c r="B259" t="str">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C259" t="str">
-        <v>236</v>
+        <v>254</v>
       </c>
       <c r="D259" t="str">
-        <v>Batul bai Johar bhai Saroda</v>
+        <v>Batul bai Mohammadhussain bhai Patra</v>
       </c>
       <c r="E259" t="str">
-        <v>30488741</v>
+        <v>20318132</v>
       </c>
       <c r="F259" t="str">
-        <v>Given</v>
+        <v>Pending</v>
       </c>
       <c r="G259" t="str">
-        <v>Ilyas</v>
+        <v/>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="str">
-        <v>1778659312652_101</v>
+        <v>1778659312652_99</v>
       </c>
       <c r="B260" t="str">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C260" t="str">
-        <v>254</v>
+        <v>236</v>
       </c>
       <c r="D260" t="str">
-        <v>Batul bai Mohammadhussain bhai Patra</v>
+        <v>Batul bai Johar bhai Saroda</v>
       </c>
       <c r="E260" t="str">
-        <v>20318132</v>
+        <v>30488741</v>
       </c>
       <c r="F260" t="str">
-        <v>Pending</v>
+        <v>Given</v>
       </c>
       <c r="G260" t="str">
-        <v/>
+        <v>Ilyas</v>
       </c>
     </row>
     <row r="261">
@@ -15601,57 +15601,66 @@
     </row>
     <row r="593">
       <c r="A593" t="str">
-        <v>1778659312652_316</v>
+        <v>1778659312652_30</v>
       </c>
       <c r="B593" t="str">
-        <v>317</v>
+        <v>31</v>
       </c>
       <c r="C593" t="str">
-        <v>235</v>
+        <v>101</v>
       </c>
       <c r="D593" t="str">
-        <v>Jumana bai Fakhruddin bhai Tarawala</v>
+        <v>Ajab bai Mufaddal bhai Bangali</v>
       </c>
       <c r="E593" t="str">
-        <v>30367675</v>
+        <v>30368206</v>
       </c>
       <c r="F593" t="str">
-        <v>Pending</v>
+        <v>Given</v>
       </c>
       <c r="G593" t="str">
-        <v/>
+        <v>Insiya ben pachlasa</v>
+      </c>
+      <c r="H593" t="str">
+        <v>23/05/2026</v>
+      </c>
+      <c r="I593" t="str">
+        <v>Saturday</v>
+      </c>
+      <c r="J593" t="str">
+        <v>12:14:22</v>
       </c>
     </row>
     <row r="594">
       <c r="A594" t="str">
-        <v>1778659312652_30</v>
+        <v>1778659312652_316</v>
       </c>
       <c r="B594" t="str">
-        <v>31</v>
+        <v>317</v>
       </c>
       <c r="C594" t="str">
-        <v>101</v>
+        <v>235</v>
       </c>
       <c r="D594" t="str">
-        <v>Ajab bai Mufaddal bhai Bangali</v>
+        <v>Jumana bai Fakhruddin bhai Tarawala</v>
       </c>
       <c r="E594" t="str">
-        <v>30368206</v>
+        <v>30367675</v>
       </c>
       <c r="F594" t="str">
         <v>Given</v>
       </c>
       <c r="G594" t="str">
-        <v>Insiya ben pachlasa</v>
+        <v>Ilyas</v>
       </c>
       <c r="H594" t="str">
-        <v>23/05/2026</v>
+        <v>28/05/2026</v>
       </c>
       <c r="I594" t="str">
-        <v>Saturday</v>
+        <v>Thursday</v>
       </c>
       <c r="J594" t="str">
-        <v>12:14:22</v>
+        <v>15:17:53</v>
       </c>
     </row>
     <row r="595">

</xml_diff>

<commit_message>
Seprate 2 Files Main distribution and Dynamic viewer
</commit_message>
<xml_diff>
--- a/backend/distribution_live_backup.xlsx
+++ b/backend/distribution_live_backup.xlsx
@@ -15648,19 +15648,10 @@
         <v>30367675</v>
       </c>
       <c r="F594" t="str">
-        <v>Given</v>
+        <v>Pending</v>
       </c>
       <c r="G594" t="str">
-        <v>Ilyas</v>
-      </c>
-      <c r="H594" t="str">
-        <v>28/05/2026</v>
-      </c>
-      <c r="I594" t="str">
-        <v>Thursday</v>
-      </c>
-      <c r="J594" t="str">
-        <v>15:17:53</v>
+        <v/>
       </c>
     </row>
     <row r="595">

</xml_diff>

<commit_message>
[2] Seprate Compnents like layouts etc
</commit_message>
<xml_diff>
--- a/backend/distribution_live_backup.xlsx
+++ b/backend/distribution_live_backup.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J781"/>
+  <dimension ref="A1:K781"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -430,6 +430,9 @@
       <c r="J1" t="str">
         <v>Update_Time</v>
       </c>
+      <c r="K1" t="str">
+        <v>Given_To</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -7129,9 +7132,21 @@
         <v>30488741</v>
       </c>
       <c r="F260" t="str">
-        <v>Given</v>
+        <v>Given to Ilyas</v>
       </c>
       <c r="G260" t="str">
+        <v>Ilyas</v>
+      </c>
+      <c r="H260" t="str">
+        <v>29/05/2026</v>
+      </c>
+      <c r="I260" t="str">
+        <v>Friday</v>
+      </c>
+      <c r="J260" t="str">
+        <v>02:04:49</v>
+      </c>
+      <c r="K260" t="str">
         <v>Ilyas</v>
       </c>
     </row>
@@ -15653,6 +15668,18 @@
       <c r="G594" t="str">
         <v/>
       </c>
+      <c r="H594" t="str">
+        <v>29/05/2026</v>
+      </c>
+      <c r="I594" t="str">
+        <v>Friday</v>
+      </c>
+      <c r="J594" t="str">
+        <v>02:05:22</v>
+      </c>
+      <c r="K594" t="str">
+        <v/>
+      </c>
     </row>
     <row r="595">
       <c r="A595" t="str">
@@ -20488,7 +20515,7 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J781"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K781"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix Dynamic Viewer issue
</commit_message>
<xml_diff>
--- a/backend/distribution_live_backup.xlsx
+++ b/backend/distribution_live_backup.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K781"/>
+  <dimension ref="A1:J781"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -430,9 +430,6 @@
       <c r="J1" t="str">
         <v>Update_Time</v>
       </c>
-      <c r="K1" t="str">
-        <v>Given_To</v>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -7117,54 +7114,42 @@
     </row>
     <row r="260">
       <c r="A260" t="str">
-        <v>1778659312652_99</v>
+        <v>1778659312652_103</v>
       </c>
       <c r="B260" t="str">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C260" t="str">
-        <v>236</v>
+        <v>1303</v>
       </c>
       <c r="D260" t="str">
-        <v>Batul bai Johar bhai Saroda</v>
+        <v>Batul bai Qutbuddin bhai Rustam</v>
       </c>
       <c r="E260" t="str">
-        <v>30488741</v>
+        <v>30366656</v>
       </c>
       <c r="F260" t="str">
-        <v>Given to Ilyas</v>
+        <v>Pending</v>
       </c>
       <c r="G260" t="str">
-        <v>Ilyas</v>
-      </c>
-      <c r="H260" t="str">
-        <v>29/05/2026</v>
-      </c>
-      <c r="I260" t="str">
-        <v>Friday</v>
-      </c>
-      <c r="J260" t="str">
-        <v>02:04:49</v>
-      </c>
-      <c r="K260" t="str">
-        <v>Ilyas</v>
+        <v/>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="str">
-        <v>1778659312652_103</v>
+        <v>1778659312652_104</v>
       </c>
       <c r="B261" t="str">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C261" t="str">
-        <v>1303</v>
+        <v>76</v>
       </c>
       <c r="D261" t="str">
-        <v>Batul bai Qutbuddin bhai Rustam</v>
+        <v>Batul bai Saifuddin bhai Doodhbhai</v>
       </c>
       <c r="E261" t="str">
-        <v>30366656</v>
+        <v>30368616</v>
       </c>
       <c r="F261" t="str">
         <v>Pending</v>
@@ -7175,19 +7160,19 @@
     </row>
     <row r="262">
       <c r="A262" t="str">
-        <v>1778659312652_104</v>
+        <v>1778659312652_105</v>
       </c>
       <c r="B262" t="str">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C262" t="str">
-        <v>76</v>
+        <v>744</v>
       </c>
       <c r="D262" t="str">
-        <v>Batul bai Saifuddin bhai Doodhbhai</v>
+        <v>Batul bai Shaikh Akbarhusain bhai Rampurwala</v>
       </c>
       <c r="E262" t="str">
-        <v>30368616</v>
+        <v>30367359</v>
       </c>
       <c r="F262" t="str">
         <v>Pending</v>
@@ -7198,80 +7183,89 @@
     </row>
     <row r="263">
       <c r="A263" t="str">
-        <v>1778659312652_105</v>
+        <v>1778659312652_106</v>
       </c>
       <c r="B263" t="str">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C263" t="str">
-        <v>744</v>
+        <v>807</v>
       </c>
       <c r="D263" t="str">
-        <v>Batul bai Shaikh Akbarhusain bhai Rampurwala</v>
+        <v>Batul bai Taiyebali bhai Bankoda</v>
       </c>
       <c r="E263" t="str">
-        <v>30367359</v>
+        <v>30367508</v>
       </c>
       <c r="F263" t="str">
-        <v>Pending</v>
+        <v>Given</v>
       </c>
       <c r="G263" t="str">
-        <v/>
+        <v>zainab ben antri</v>
+      </c>
+      <c r="H263" t="str">
+        <v>18/05/2026</v>
+      </c>
+      <c r="I263" t="str">
+        <v>Monday</v>
+      </c>
+      <c r="J263" t="str">
+        <v>11:50:34</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="str">
-        <v>1778659312652_106</v>
+        <v>1778659312652_6</v>
       </c>
       <c r="B264" t="str">
-        <v>107</v>
+        <v>7</v>
       </c>
       <c r="C264" t="str">
-        <v>807</v>
+        <v>7</v>
       </c>
       <c r="D264" t="str">
-        <v>Batul bai Taiyebali bhai Bankoda</v>
+        <v>Abbas bhai Alihusain bhai Sihjee</v>
       </c>
       <c r="E264" t="str">
-        <v>30367508</v>
+        <v>20435003</v>
       </c>
       <c r="F264" t="str">
         <v>Given</v>
       </c>
       <c r="G264" t="str">
-        <v>zainab ben antri</v>
+        <v>Ajab ben Khand</v>
       </c>
       <c r="H264" t="str">
-        <v>18/05/2026</v>
+        <v>21/05/2026</v>
       </c>
       <c r="I264" t="str">
-        <v>Monday</v>
+        <v>Thursday</v>
       </c>
       <c r="J264" t="str">
-        <v>11:50:34</v>
+        <v>10:25:43</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="str">
-        <v>1778659312652_6</v>
+        <v>1778659312652_335</v>
       </c>
       <c r="B265" t="str">
-        <v>7</v>
+        <v>336</v>
       </c>
       <c r="C265" t="str">
-        <v>7</v>
+        <v>1197</v>
       </c>
       <c r="D265" t="str">
-        <v>Abbas bhai Alihusain bhai Sihjee</v>
+        <v>Khanali bhai Mohammadhussain bhai Hedari</v>
       </c>
       <c r="E265" t="str">
-        <v>20435003</v>
+        <v>20414120</v>
       </c>
       <c r="F265" t="str">
         <v>Given</v>
       </c>
       <c r="G265" t="str">
-        <v>Ajab ben Khand</v>
+        <v/>
       </c>
       <c r="H265" t="str">
         <v>21/05/2026</v>
@@ -7280,39 +7274,30 @@
         <v>Thursday</v>
       </c>
       <c r="J265" t="str">
-        <v>10:25:43</v>
+        <v>11:08:30</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="str">
-        <v>1778659312652_335</v>
+        <v>1778659312652_99</v>
       </c>
       <c r="B266" t="str">
-        <v>336</v>
+        <v>100</v>
       </c>
       <c r="C266" t="str">
-        <v>1197</v>
+        <v>236</v>
       </c>
       <c r="D266" t="str">
-        <v>Khanali bhai Mohammadhussain bhai Hedari</v>
+        <v>Batul bai Johar bhai Saroda</v>
       </c>
       <c r="E266" t="str">
-        <v>20414120</v>
+        <v>30488741</v>
       </c>
       <c r="F266" t="str">
         <v>Given</v>
       </c>
       <c r="G266" t="str">
-        <v/>
-      </c>
-      <c r="H266" t="str">
-        <v>21/05/2026</v>
-      </c>
-      <c r="I266" t="str">
-        <v>Thursday</v>
-      </c>
-      <c r="J266" t="str">
-        <v>11:08:30</v>
+        <v>Ilyas</v>
       </c>
     </row>
     <row r="267">
@@ -15668,18 +15653,6 @@
       <c r="G594" t="str">
         <v/>
       </c>
-      <c r="H594" t="str">
-        <v>29/05/2026</v>
-      </c>
-      <c r="I594" t="str">
-        <v>Friday</v>
-      </c>
-      <c r="J594" t="str">
-        <v>02:05:22</v>
-      </c>
-      <c r="K594" t="str">
-        <v/>
-      </c>
     </row>
     <row r="595">
       <c r="A595" t="str">
@@ -20515,7 +20488,7 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K781"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J781"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>